<commit_message>
Recover partial daily sync (2026-07-08, interrupted mid-run)
</commit_message>
<xml_diff>
--- a/Investment_Research_Dashboard.xlsx
+++ b/Investment_Research_Dashboard.xlsx
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="NewsTable" displayName="NewsTable" ref="A1:I259" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="NewsTable" displayName="NewsTable" ref="A1:I305" headerRowCount="1">
   <autoFilter ref="A1:I11"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Date"/>
@@ -338,7 +338,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="NarrativeTable" displayName="NarrativeTable" ref="A1:P27" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="NarrativeTable" displayName="NarrativeTable" ref="A1:P36" headerRowCount="1">
   <autoFilter ref="A1:P2"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Ticker"/>
@@ -652,7 +652,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -668,7 +668,7 @@
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="60" customWidth="1" min="17" max="17"/>
     <col width="21" customWidth="1" min="18" max="18"/>
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="R2" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="3">
@@ -903,7 +903,7 @@
         </is>
       </c>
       <c r="R3" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="4">
@@ -933,16 +933,16 @@
         </is>
       </c>
       <c r="F4" s="8" t="n">
-        <v>196.9</v>
+        <v>196.93</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>4768875413504</v>
+        <v>4769841152000</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>30.151623</v>
+        <v>30.157732</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>15.424904</v>
+        <v>15.428029</v>
       </c>
       <c r="J4" s="9" t="n">
         <v>0.5996</v>
@@ -969,11 +969,11 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>NVIDIA is a rare combination of hypergrowth and exceptional profitability: ~85% YoY revenue growth, ~75% gross margins, ~77% ROIC, ~$49B quarterly FCF, and a near-debt-free balance sheet. At a forward...</t>
+          <t>NVIDIA is a rare combination of hypergrowth and exceptional profitability: ~85% YoY revenue growth, ~75% gross margins, ~77% ROIC, ~$49B quarterly FCF, and a near-debt-free balance sheet. At forward P...</t>
         </is>
       </c>
       <c r="R4" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="5">
@@ -1003,16 +1003,16 @@
         </is>
       </c>
       <c r="F5" s="8" t="n">
-        <v>435.605</v>
+        <v>432.57</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>2259253985280</v>
+        <v>2243513024512</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>37.812935</v>
+        <v>37.549477</v>
       </c>
       <c r="I5" s="9" t="n">
-        <v>21.469807</v>
+        <v>21.32022</v>
       </c>
       <c r="J5" s="9" t="n">
         <v>1.4213</v>
@@ -1039,11 +1039,11 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>TSMC is a best-in-class business trading at a fair-but-not-cheap valuation. The core thesis: it is the indispensable manufacturer of the leading-edge chips powering the AI buildout, with a moat eviden...</t>
+          <t>TSMC is a best-in-class business at a fair-but-not-cheap valuation, and nothing this week alters that. It is the indispensable manufacturer of leading-edge AI chips, with a moat evidenced by hard numb...</t>
         </is>
       </c>
       <c r="R5" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="6">
@@ -1073,16 +1073,16 @@
         </is>
       </c>
       <c r="F6" s="8" t="n">
-        <v>371.05</v>
+        <v>370.78</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>1765300109312</v>
+        <v>1764015603712</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>61.63621</v>
+        <v>61.591362</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>19.13045</v>
+        <v>19.11653</v>
       </c>
       <c r="J6" s="9" t="n">
         <v>0.4052</v>
@@ -1109,11 +1109,11 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Broadcom is a high-quality compounder benefiting from a genuine AI-driven inflection, evidenced by revenue reaccelerating to ~48% YoY, operating margins expanding to ~49%, ~46% FCF margins, and improv...</t>
+          <t>Broadcom is a high-quality compounder benefiting from a genuine AI-driven inflection: revenue reaccelerating to ~48% YoY, operating margins expanding to ~49%, ~46% FCF margins, and improving returns o...</t>
         </is>
       </c>
       <c r="R6" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="7">
@@ -1143,16 +1143,16 @@
         </is>
       </c>
       <c r="F7" s="8" t="n">
-        <v>337.46</v>
+        <v>339.22</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>904227848192</v>
+        <v>908943818752</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>16.146412</v>
+        <v>16.230623</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>14.146645</v>
+        <v>14.205538</v>
       </c>
       <c r="J7" s="9" t="n">
         <v>1.7686</v>
@@ -1179,11 +1179,11 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>JPMorgan is a best-in-class, diversified megabank that consistently earns mid-teens returns on equity, compounds tangible book value through cycles, and returns substantial capital to shareholders. Th...</t>
+          <t>JPMorgan is a best-in-class, diversified megabank that consistently earns mid-teens ROE, compounds tangible book value through cycles, and returns substantial capital via dividends and buybacks. The l...</t>
         </is>
       </c>
       <c r="R7" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="8">
@@ -1213,16 +1213,16 @@
         </is>
       </c>
       <c r="F8" s="8" t="n">
-        <v>350.09</v>
+        <v>352.2</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>665781469184</v>
+        <v>669794172928</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>30.52223</v>
+        <v>30.70619</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>23.542742</v>
+        <v>23.684635</v>
       </c>
       <c r="J8" s="9" t="n">
         <v>1.5893</v>
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c r="R8" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="9">
@@ -1283,19 +1283,19 @@
         </is>
       </c>
       <c r="F9" s="8" t="n">
-        <v>532.5551</v>
+        <v>531.62</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>470557097984</v>
+        <v>469730852864</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>30.837006</v>
+        <v>30.78286</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>23.372032</v>
+        <v>23.332333</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>1.6596</v>
+        <v>1.6403</v>
       </c>
       <c r="K9" s="5" t="n">
         <v>0.006500000000000001</v>
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="R9" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="10">
@@ -1353,16 +1353,16 @@
         </is>
       </c>
       <c r="F10" s="8" t="n">
-        <v>245.7408</v>
+        <v>245.98</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>2643344490496</v>
+        <v>2646033825792</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>31.83031</v>
+        <v>31.862694</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>24.81492</v>
+        <v>24.840168</v>
       </c>
       <c r="J10" s="9" t="n">
         <v>1.8344</v>
@@ -1387,11 +1387,11 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Amazon is a high-quality, multi-engine compounder whose profitability has structurally improved (operating margins now 11-13% vs low single digits historically) even as it grows revenue ~17% at massiv...</t>
+          <t>Amazon is a high-quality, multi-engine compounder whose profitability has structurally improved (operating margins now 11-13% vs low single digits historically) while still growing revenue ~17% at mas...</t>
         </is>
       </c>
       <c r="R10" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="11">
@@ -1421,16 +1421,16 @@
         </is>
       </c>
       <c r="F11" s="8" t="n">
-        <v>282.045</v>
+        <v>282.21</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>200394637312</v>
+        <v>200511848448</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>23.251856</v>
+        <v>23.265457</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>19.833845</v>
+        <v>19.845446</v>
       </c>
       <c r="J11" s="9" t="n">
         <v>2.5635</v>
@@ -1457,11 +1457,11 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>McDonald's is a wide-moat, capital-light, cash-generative franchise business trading at a full-but-fair valuation after a ~17% pullback from its high. The Q1 2026 data confirms the business is executi...</t>
+          <t>McDonald's is a wide-moat, capital-light, cash-generative franchise business trading at a full-but-fair valuation after a ~17% pullback. Q1 2026 confirms execution -- ~9.4% revenue growth and ~7% EPS ...</t>
         </is>
       </c>
       <c r="R11" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="12">
@@ -1491,16 +1491,16 @@
         </is>
       </c>
       <c r="F12" s="8" t="n">
-        <v>43.02</v>
+        <v>43.21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>63707762688</v>
+        <v>63989129216</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>20.485716</v>
+        <v>20.57619</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>18.10469</v>
+        <v>18.543713</v>
       </c>
       <c r="J12" s="9" t="n">
         <v>1.5389</v>
@@ -1512,8 +1512,18 @@
       <c r="M12" s="5" t="n"/>
       <c r="N12" s="5" t="n"/>
       <c r="O12" s="9" t="n"/>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Fairly Valued</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Nike is a high-quality, dominant brand undergoing a self-inflicted turnaround that appears to be inflecting, trading near multi-year lows at a below-historical valuation. The core thesis is a margin-r...</t>
+        </is>
+      </c>
       <c r="R12" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="13">
@@ -3014,6 +3024,105 @@
     <cfRule type="cellIs" priority="90" operator="equal" dxfId="2">
       <formula>"Fairly Valued"</formula>
     </cfRule>
+    <cfRule type="cellIs" priority="91" operator="equal" dxfId="0">
+      <formula>"Undervalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="92" operator="equal" dxfId="1">
+      <formula>"Overvalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="93" operator="equal" dxfId="2">
+      <formula>"Fairly Valued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="94" operator="equal" dxfId="0">
+      <formula>"Undervalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="95" operator="equal" dxfId="1">
+      <formula>"Overvalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="96" operator="equal" dxfId="2">
+      <formula>"Fairly Valued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="97" operator="equal" dxfId="0">
+      <formula>"Undervalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="98" operator="equal" dxfId="1">
+      <formula>"Overvalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="99" operator="equal" dxfId="2">
+      <formula>"Fairly Valued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="100" operator="equal" dxfId="0">
+      <formula>"Undervalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="101" operator="equal" dxfId="1">
+      <formula>"Overvalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="102" operator="equal" dxfId="2">
+      <formula>"Fairly Valued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="103" operator="equal" dxfId="0">
+      <formula>"Undervalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="104" operator="equal" dxfId="1">
+      <formula>"Overvalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="105" operator="equal" dxfId="2">
+      <formula>"Fairly Valued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="106" operator="equal" dxfId="0">
+      <formula>"Undervalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="107" operator="equal" dxfId="1">
+      <formula>"Overvalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="108" operator="equal" dxfId="2">
+      <formula>"Fairly Valued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="109" operator="equal" dxfId="0">
+      <formula>"Undervalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="110" operator="equal" dxfId="1">
+      <formula>"Overvalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="111" operator="equal" dxfId="2">
+      <formula>"Fairly Valued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="112" operator="equal" dxfId="0">
+      <formula>"Undervalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="113" operator="equal" dxfId="1">
+      <formula>"Overvalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="114" operator="equal" dxfId="2">
+      <formula>"Fairly Valued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="115" operator="equal" dxfId="0">
+      <formula>"Undervalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="116" operator="equal" dxfId="1">
+      <formula>"Overvalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="117" operator="equal" dxfId="2">
+      <formula>"Fairly Valued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="118" operator="equal" dxfId="0">
+      <formula>"Undervalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="119" operator="equal" dxfId="1">
+      <formula>"Overvalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="120" operator="equal" dxfId="2">
+      <formula>"Fairly Valued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="121" operator="equal" dxfId="0">
+      <formula>"Undervalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="122" operator="equal" dxfId="1">
+      <formula>"Overvalued"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="123" operator="equal" dxfId="2">
+      <formula>"Fairly Valued"</formula>
+    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -3029,7 +3138,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -3608,7 +3717,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
@@ -3845,13 +3954,13 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>196.9</v>
+        <v>196.93</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>4768875413504</v>
+        <v>4769841152000</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>4691951878144</v>
@@ -3860,19 +3969,19 @@
         <v>24221000000</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>30.151623</v>
+        <v>30.157732</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>15.424904</v>
+        <v>15.428029</v>
       </c>
       <c r="I4" s="9" t="n">
         <v>0.5996</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>18.813742</v>
+        <v>18.816608</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>24.397783</v>
+        <v>24.402725</v>
       </c>
       <c r="L4" s="9" t="n">
         <v>18.509</v>
@@ -3903,13 +4012,13 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>435.605</v>
+        <v>432.57</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>2259253985280</v>
+        <v>2243513024512</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>16497778884608</v>
@@ -3918,19 +4027,19 @@
         <v>5186474013</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>37.812935</v>
+        <v>37.549477</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>21.469807</v>
+        <v>21.32022</v>
       </c>
       <c r="I5" s="9" t="n">
         <v>1.4213</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0.5505133</v>
+        <v>0.5466777</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>98.05056</v>
+        <v>97.36741000000001</v>
       </c>
       <c r="L5" s="9" t="n">
         <v>4.02</v>
@@ -3961,13 +4070,13 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>371.05</v>
+        <v>370.78</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1765300109312</v>
+        <v>1764015603712</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>1824138199040</v>
@@ -3976,19 +4085,19 @@
         <v>4757580198</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>61.63621</v>
+        <v>61.591362</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>19.13045</v>
+        <v>19.11653</v>
       </c>
       <c r="I6" s="9" t="n">
         <v>0.4052</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>23.392303</v>
+        <v>23.375282</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>20.132935</v>
+        <v>20.118284</v>
       </c>
       <c r="L6" s="9" t="n">
         <v>24.172</v>
@@ -4019,13 +4128,13 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>337.46</v>
+        <v>339.22</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>904227848192</v>
+        <v>908943818752</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>663828627456</v>
@@ -4034,19 +4143,19 @@
         <v>2679511418</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>16.146412</v>
+        <v>16.230623</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>14.146645</v>
+        <v>14.205538</v>
       </c>
       <c r="I7" s="9" t="n">
         <v>1.7686</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>5.209916</v>
+        <v>5.237088</v>
       </c>
       <c r="K7" s="9" t="n">
-        <v>2.628623</v>
+        <v>2.6423326</v>
       </c>
       <c r="L7" s="9" t="n">
         <v>3.825</v>
@@ -4075,13 +4184,13 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>350.09</v>
+        <v>352.2</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>665781469184</v>
+        <v>669794172928</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>683806818304</v>
@@ -4090,19 +4199,19 @@
         <v>1659709932</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>30.52223</v>
+        <v>30.70619</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>23.542742</v>
+        <v>23.684635</v>
       </c>
       <c r="I8" s="9" t="n">
         <v>1.5893</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>15.473574</v>
+        <v>15.5668335</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>18.779636</v>
+        <v>18.892822</v>
       </c>
       <c r="L8" s="9" t="n">
         <v>15.893</v>
@@ -4133,13 +4242,13 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>532.5551</v>
+        <v>531.62</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>470557097984</v>
+        <v>469730852864</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>481782562816</v>
@@ -4148,19 +4257,19 @@
         <v>877036230</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>30.837006</v>
+        <v>30.78286</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>23.372032</v>
+        <v>23.332333</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>1.6596</v>
+        <v>1.6403</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>13.86479</v>
+        <v>13.840445</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>70.29501999999999</v>
+        <v>70.17158999999999</v>
       </c>
       <c r="L9" s="9" t="n">
         <v>14.196</v>
@@ -4191,40 +4300,40 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>245.7408</v>
+        <v>245.98</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>2643344490496</v>
+        <v>2646033825792</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>2718906712064</v>
+        <v>2738484674560</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>10757109436</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>31.83031</v>
+        <v>31.862694</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>24.81492</v>
+        <v>24.840168</v>
       </c>
       <c r="I10" s="9" t="n">
         <v>1.8344</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>3.5588934</v>
+        <v>3.562358</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>5.979851</v>
+        <v>5.9859343</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>3.66</v>
+        <v>3.687</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>17.444</v>
+        <v>17.57</v>
       </c>
       <c r="N10" s="5" t="n"/>
       <c r="O10" s="9" t="n">
@@ -4247,13 +4356,13 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>282.045</v>
+        <v>282.21</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>200394637312</v>
+        <v>200511848448</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>252311388160</v>
@@ -4262,19 +4371,19 @@
         <v>710505859</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>23.251856</v>
+        <v>23.265457</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>19.833845</v>
+        <v>19.845446</v>
       </c>
       <c r="I11" s="9" t="n">
         <v>2.5635</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>7.301415</v>
+        <v>7.3056855</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>-155.82597</v>
+        <v>-155.91713</v>
       </c>
       <c r="L11" s="9" t="n">
         <v>9.193</v>
@@ -4305,40 +4414,40 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>46210</v>
+        <v>46211</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>43.02</v>
+        <v>43.21</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>63707762688</v>
+        <v>63989129216</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>66261884928</v>
+        <v>66069147648</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>1199499281</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>20.485716</v>
+        <v>20.57619</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>18.10469</v>
+        <v>18.543713</v>
       </c>
       <c r="I12" s="9" t="n">
         <v>1.5389</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>1.3730713</v>
+        <v>1.3791355</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>4.290844</v>
+        <v>4.3097944</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>1.428</v>
+        <v>1.424</v>
       </c>
       <c r="M12" s="9" t="n">
-        <v>14.609</v>
+        <v>14.567</v>
       </c>
       <c r="N12" s="5" t="n">
         <v>0.0378</v>
@@ -5347,7 +5456,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q174"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
@@ -5359,7 +5468,7 @@
     <col width="23" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
@@ -13141,7 +13250,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Y174"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
@@ -25650,8 +25759,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I259"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:I305"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
@@ -37321,6 +37430,2076 @@
         </is>
       </c>
     </row>
+    <row r="260">
+      <c r="A260" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>DeepSeek looks to reduce reliance on Nvidia with own AI chip</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Yahoo Finance Video</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/video/deepseek-looks-to-reduce-reliance-on-nvidia-with-own-ai-chip-203313261.html</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>A major AI customer building its own chips signals rising competitive pressure that could erode Nvidia's dominant market share over time.</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>2 Beaten-Down Artificial Intelligence (AI) Stocks That Will Surge at Least 40% Over the Next Year, According to Wall Street</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/investing/2026/07/07/beaten-down-artificial-intelligence-ai-stocks/</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Analyst optimism on beaten-down AI names signals potential sector-wide upside, but NVDA may not be among the specific stocks featured.</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>SpaceX Has Joined the Nasdaq-100. Here's What That Means for Index Investors</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/investing/2026/07/07/spacex-has-joined-the-nasdaq-100-heres-what-that-means-for-index-investors/</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Nasdaq-100 composition changes have negligible direct impact on NVDA fundamentals, though index reweighting could marginally affect passive fund flows into the stock.</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Why Fiserv Stock Topped the Market Today</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/investing/2026/07/07/why-fiserv-stock-topped-the-market-today/</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>This headline concerns Fiserv's business unit sale and has no material relevance to NVDA's fundamentals or outlook.</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Why Sandisk Stock Jumped 34% in June</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/investing/2026/07/07/why-sandisk-stock-jumped-34-in-june/</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>Strong memory chip demand signals healthy AI infrastructure spending, supporting sustained demand for NVDA's GPUs that rely on high-bandwidth memory.</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Microsoft Looks to Make a Major Reset as It Says This Area of Its Business "Is Not Healthy"</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/investing/2026/07/07/microsoft-looks-to-make-a-major-reset-as-it-says-t/</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>Microsoft's restructuring is company-specific and only tangentially affects NVDA; unclear if AI spending or GPU demand shifts materially.</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Nervous About the Stock Market? These 7 Words From Warren Buffett Might Change Your Mind.</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/investing/2026/07/07/nervous-about-stock-market-7-words-warren-buffett/</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>Reinforces a buy-during-fear mindset, suggesting NVDA holders should stay disciplined and view market dips as long-term opportunities.</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Hormuz Tolls Are Just the Beginning: The World’s Busiest Shipping Route Could Be Next</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>https://247wallst.com/investing/2026/07/07/hormuz-tolls-are-just-the-beginning-the-worlds-busiest-shipping-route-could-be-next/</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Geopolitical shipping disruptions could raise supply chain costs and delay NVDA hardware shipments, though impact on the company is indirect.</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Amazon Stocks Climbs As AI Push Drives $25 Billion Bond Sale</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>https://www.investors.com/news/technology/amazon-stock-25-billion-bond-ai-costs-rising/?src=A00220&amp;yptr=yahoo</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Amazon's $25B bond-funded AI infrastructure buildout signals continued hyperscaler capex, sustaining strong demand for NVDA's data center GPUs.</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Robinhood Is Making a Comeback. Should You Buy the Stock?</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/investing/2026/07/07/robinhood-is-making-a-comeback-should-you-buy-the/</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>NVIDIA Corporation</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>This headline concerns Robinhood, not NVDA, and has no direct relevance to NVDA's fundamentals or long-term investment thesis.</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>DeepSeek looks to reduce reliance on Nvidia with own AI chip</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Yahoo Finance Video</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/video/deepseek-looks-to-reduce-reliance-on-nvidia-with-own-ai-chip-203313261.html</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Taiwan Semiconductor Manufacturing Company</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>DeepSeek's custom AI chip would likely be fabricated by TSMC, expanding its foundry customer base beyond Nvidia as chip design diversifies.</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Samsung saw a record quarter, but it's not enough for investors. Here's why.</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Yahoo Finance Video</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/video/samsung-saw-a-record-quarter-but-its-not-enough-for-investors-heres-why-203148500.html</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Taiwan Semiconductor Manufacturing Company</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Memory sector volatility from Samsung's results signals broader semiconductor demand dynamics that could indirectly affect TSM's foundry outlook.</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>This Semiconductor ETF Is Up 58% This Year and Doesn’t Own TSMC</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>https://247wallst.com/investing/etf/2026/07/07/this-semiconductor-etf-is-up-58-this-year-and-doesnt-own-tsmc/</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Taiwan Semiconductor Manufacturing Company</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>The article highlights TSM's central role fabricating chips for AI designers, reinforcing its indispensability even when excluded from a fabless-focused ETF.</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Up 102% in 2026, This Chip ETF Mysteriously Avoids Taiwan Semiconductor</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>https://247wallst.com/investing/etf/2026/07/07/up-102-in-2026-this-chip-etf-mysteriously-avoids-taiwan-semiconductor/</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Taiwan Semiconductor Manufacturing Company</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>TSM's exclusion from a top-performing chip ETF is a fund-construction quirk, not a reflection of the company's underlying business fundamentals.</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Bank of America Analyst: AI Is Becoming “Deeply Embedded in Enterprise Workflows” as AI Spending Could Reach $1.5 Trillion</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>https://247wallst.com/investing/2026/07/07/bank-of-america-analyst-ai-is-becoming-deeply-embedded-in-enterprise-workflows-as-ai-spending-could-reach-1-5-trillion/</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Taiwan Semiconductor Manufacturing Company</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Accelerating enterprise AI adoption and massive projected spending signal sustained long-term demand for TSM's advanced chip manufacturing.</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Wall Street tech analyst explains why investors should look past Samsung selloff</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Investing.com</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/wall-street-tech-analyst-explains-163203461.html</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Taiwan Semiconductor Manufacturing Company</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Analyst frames the semiconductor selloff as technical momentum unwind rather than fundamental weakness, suggesting TSM's downside is temporary and buyable.</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>A Circuit Board Problem Just Delayed Nvidia’s Next AI System to 2028 And Chip Stocks Are Already Feeling the Fallout</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>https://247wallst.com/investing/2026/07/07/a-circuit-board-problem-just-delayed-nvidias-next-ai-system-to-2028-and-chip-stocks-are-already-feeling-the-fallout/</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>A delayed Nvidia AI system could dampen near-term demand for Broadcom's networking and custom chips tied to AI rack deployments.</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Semtech, Power Integrations, Amkor, Entegris, and Kulicke and Soffa Stocks Trade Down, What You Need To Know</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>StockStory</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/semtech-power-integrations-amkor-entegris-194552439.html</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Semiconductor sector weakness and DeepSeek's in-house AI chip development signal competitive pressures that could affect AVGO's AI chip demand outlook.</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>FormFactor, Penguin Solutions, Western Digital, Applied Materials, and KLA Corporation Shares Plummet, What You Need To Know</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>StockStory</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/formfactor-penguin-solutions-western-digital-193752825.html</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>DeepSeek developing its own AI inference chip signals potential competitive threat to Broadcom's custom AI accelerator business over the long term.</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>DeepSeek Reportedly Develops AI Chip as Nvidia Shares Drop 2.2%</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>GuruFocus.com</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/technology/ai/articles/deepseek-reportedly-develops-ai-chip-192001405.html</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Rising custom AI silicon efforts by firms like DeepSeek validate Broadcom's ASIC design business, though it also intensifies competition for AI chip market share.</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Broadcom Stock Drops After Bank Downgrades AI Chip Giant on Valuation</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>GuruFocus.com</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/broadcom-stock-drops-bank-downgrades-184733964.html</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>A valuation-based downgrade signals near-term price concerns but doesn't undermine Broadcom's long-term AI growth fundamentals or business strength.</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Bank of America Analyst: AI Is Becoming “Deeply Embedded in Enterprise Workflows” as AI Spending Could Reach $1.5 Trillion</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>https://247wallst.com/investing/2026/07/07/bank-of-america-analyst-ai-is-becoming-deeply-embedded-in-enterprise-workflows-as-ai-spending-could-reach-1-5-trillion/</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Broadcom Inc.</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Sustained AI infrastructure spending growth supports long-term demand for AVGO's custom AI chips and networking products.</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>SpaceX stock drops below IPO opening price despite flood of bullish Wall Street ratings</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/article/spacex-stock-drops-below-ipo-opening-price-despite-flood-of-bullish-wall-street-ratings-153809443.html</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>This headline concerns SpaceX, not JPM, and has no material relevance to a long-term JPMorgan investor.</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Fiserv Stock Rises on Report Big U.S. Banks Explore Buying Its Debit Card Network</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Barrons.com</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>https://www.barrons.com/articles/fiserv-stock-jpmorgan-wells-fargo-debit-card-73e8fb35?siteid=yhoof2&amp;yptr=yahoo</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>JPM exploring a joint acquisition of a debit network could reduce reliance on third-party processors and strengthen payments infrastructure control.</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Avaada Seeks $750 Million Refinancing as India Clean-Energy Push Accelerates</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>GuruFocus.com</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/energy/articles/avaada-seeks-750-million-refinancing-191620378.html</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>This deal signals fee opportunities in emerging-market clean-energy financing, but no direct JPM involvement is indicated, limiting relevance.</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>JPMorgan Cuts Yuan Bets Despite 3% Gain, Eyes New Currency Winners</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>GuruFocus.com</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/currencies/articles/jpmorgan-cuts-yuan-bets-despite-185641555.html</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>JPM's asset management arm is actively repositioning FX strategies, reflecting tactical currency views rather than material impact on the firm's fundamentals.</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Fiserv Explores Sale of Debit Network</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>GuruFocus.com</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/fiserv-explores-sale-debit-network-182705349.html</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>A potential STAR Network acquisition could expand JPM's payments infrastructure and merchant reach, but financial impact depends on deal terms.</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Acquisition</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Which Small Cap ETF Is the Better Buy in 2026? iShares and JPMorgan Have Compelling Offerings</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/coverage/etfs/2026/07/07/which-small-cap-etf-is-the-better-buy-in-2026-ishares-and-jpmorgan-have-compelling-offerings/</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Highlights JPMorgan's competitive ETF offerings, showing its asset management arm can attract inflows and diversify revenue beyond banking.</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Nvidia-Backed Nscale Secures $900 Million Credit Facility for AI Expansion</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>GuruFocus.com</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/technology/ai/articles/nvidia-backed-nscale-secures-900-170032178.html</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>This headline concerns Nvidia and Nscale AI financing with no clear connection to JPM's business or investment outlook.</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Major US Banks' Second-Quarter Earnings Poised for Upside, BofA Says</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>MT Newswires</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/major-us-banks-apos-second-165554609.html</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>JPMorgan Chase &amp; Co.</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Strong capital markets recovery could signal sustained revenue diversification, benefiting JPM's earnings resilience beyond traditional lending income.</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Circle's USDC now runs 70% of the stablecoin volume</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Yahoo Finance Video</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/video/circles-usdc-now-runs-70-183000137.html</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Growing stablecoin adoption could disintermediate traditional card networks like Visa, posing a long-term competitive threat to payment volumes.</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>DDSC Brings Regulated Dirham Stablecoin to UAE Exchanges</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>BeInCrypto</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>https://beincrypto.com/uae-dirham-stablecoin-ddsc-exchange-access/</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Regulated dirham stablecoins could bypass card networks for payments, posing a long-term disintermediation risk to Visa's transaction volumes in the region.</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Is Visa (V) Undervalued After Its AI Payments Push And Stablecoin Moves?</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Simply Wall St.</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/visa-v-undervalued-ai-payments-211813162.html</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Visa's expansion into agentic commerce and stablecoin payments signals proactive adaptation to emerging technologies, potentially defending its network dominance and long-term growth.</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Dow Jones Payments Leader Visa Breaks Out; Arista Networks Eyes Buy Point</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Investor's Business Daily</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>https://www.investors.com/stock-lists/stocks-near-a-buy-zone/dow-jones-visa-stock-v-buy-zone-investing-markets/?src=A00220&amp;yptr=yahoo</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Technical breakout signals strong price momentum and investor confidence, though it reflects trading dynamics rather than fundamental business developments for Visa.</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Visa vs Coinbase: Two Different Economic Playbooks But One Winner</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>https://247wallst.com/investing/2026/07/07/visa-vs-coinbase-two-different-economic-playbooks-but-one-winner/</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Visa Inc.</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Visa's steady payment volumes and 15% revenue growth demonstrate resilience against crypto disruption, reinforcing its durable competitive moat.</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Mastercard (MA) Joins Open USD Stablecoin, Is The Stock Still Cheap?</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Simply Wall St.</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/mastercard-ma-joins-open-usd-171402878.html</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Mastercard Incorporated</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Mastercard's stablecoin adoption and buyback signal proactive positioning in digital payments, potentially defending its network relevance amid crypto disruption.</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>DeepSeek looks to reduce reliance on Nvidia with own AI chip</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Yahoo Finance Video</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/video/deepseek-looks-to-reduce-reliance-on-nvidia-with-own-ai-chip-203313261.html</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>DeepSeek's custom chip signals broader industry shift toward AI hardware independence, indirectly validating Amazon's own Trainium/Inferentia investments amid Nvidia reliance concerns.</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Roku vs. Sirius XM: Which Media Stock Is a Better Buy in 2026?</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/coverage/better-buy/2026/07/07/roku-vs-sirius-xm-which-media-stock-is-a-better-buy-in-2026/</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>This headline compares Roku and Sirius XM, with no direct relevance to Amazon's business or investment thesis.</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Nasdaq Slides Nearly 2% As Higher Treasury Yields, Soaring Oil Prices Pressure Tech And Chip Stocks — META, AMZN, SPCX, MSFT In Focus</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Stocktwits</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>https://stocktwits.com/news-articles/markets/equity/nasdaq-slides-nearly-2-as-higher-treasury-yields-soaring-oil-prices-pressure-tech-and-chip-stocks-meta-amzn-spcx-msft-in-focus/cZmlDzSR7ZV</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Broad macro pressures like rising yields and oil prices weigh on tech valuations, but AMZN's long-term fundamentals remain unaffected by short-term sentiment.</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Amazon's Stock Is Historically Cheap. Now Is Your Perfect Buying Opportunity</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/investing/2026/07/07/amazons-stock-is-historically-cheap-now-is-your-pe/</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Anticipated AWS growth combined with a relatively low valuation could offer long-term investors an attractive entry point with upside potential.</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Top Analyst Reports for Amazon.com, Walmart &amp; American Express</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Zacks</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/top-analyst-reports-amazon-com-211500537.html</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>Amazon's AI investments and global diversification drive long-term growth, though elevated spending and competition may pressure near-term margins.</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Trump's $1.4 Billion Crypto Haul Draws Fresh Investor Scrutiny</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>GuruFocus.com</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>https://www.yahoo.com/news/politics/articles/trumps-1-4-billion-crypto-195905371.html</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>This headline concerns Trump's personal crypto ventures and has no material connection to Amazon's business or fundamentals.</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Amazon Plans $25 Billion Bond Sale</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>GuruFocus.com</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/amazon-plans-25-billion-bond-192227995.html</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>Debt-funded AI and data-center investment signals aggressive capacity expansion, though rising leverage adds interest costs and execution risk to future returns.</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Amazon's AI Spending Push Hits Bond Market</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>GuruFocus.com</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.com/markets/stocks/articles/amazons-ai-spending-push-hits-191559609.html</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Amazon.com, Inc.</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>Debt-funded AI capex signals aggressive investment that could pressure near-term free cash flow while betting on long-term cloud and AI growth.</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>The Dividend Growth Snowball: How Modest Income Today Can Become Serious Income Later</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>24/7 Wall St.</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>https://247wallst.com/personal-finance/2026/07/07/the-dividend-growth-snowball-how-modest-income-today-can-become-serious-income-later/</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>McDonald's Corporation</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>MCD</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>MCD's consistent dividend growth history makes it a candidate for compounding income that outpaces high-yield alternatives over long holding periods.</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="10" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>McDonald's Franchise Owners Make A Surprising Amount Of Money</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Money Digest</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>https://www.moneydigest.com/1788834/how-much-money-does-mcdonalds-franchise-owners-make/</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>McDonald's Corporation</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>MCD</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Franchisee profitability affects franchise system health, expansion appetite, and MCD's royalty-based revenue stream stability over the long term.</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -37335,8 +39514,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:P36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
@@ -39362,6 +41541,672 @@
         <v>78</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>NVIDIA remains an exceptional business at the center of the AI data center buildout, with financials essentially unchanged from the prior day's analysis. The latest reported quarter (period ending 2026-04-30) showed ~$81.6B in revenue (~85% YoY growth), ~75% gross margin, mid-60s% operating margin, ~$48.6B free cash flow, and a near-debt-free balance sheet (D/E ~0.06). Returns on capital are among the highest of any large-cap (ROIC ~77%, ROE ~82% per prior derivation). The stock at $196.93 trades at ~30x trailing and ~15.4x forward earnings with a PEG below 0.6 -- undemanding for the growth trajectory, though price-to-sales ~19 and EV/EBITDA ~28 are rich in absolute terms and depend on demand durability. The central debate is unchanged: not whether NVIDIA is a great business (the data confirms it is), but whether the hyperscaler capex supercycle is durable and how fast custom silicon and AMD erode its position. Today's news adds one incrementally negative competitive data point (DeepSeek building its own chip) balanced against fresh positive signals on hyperscaler capex (Amazon's $25B AI bond, strong memory demand). None of this materially changes the thesis.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Only one calendar day has elapsed since the prior writeup and no new financial data was released, so there is no material change to fundamentals. The one incrementally meaningful news item is a report that DeepSeek -- a significant AI customer -- is developing its own AI chip to reduce Nvidia reliance. This is thematically consistent with the previously noted customer-diversification trend (Turing/AMD, TPUs) rather than a new category of risk; it adds another data point to the 'largest customers are motivated to build alternatives' bear narrative but is too small and too early to quantify. Offsetting this, two news items reinforce the bull side of demand durability: Amazon's $25B bond-funded AI infrastructure buildout signals continued hyperscaler capex, and strong memory-chip (Sandisk) demand corroborates healthy AI infrastructure spending that underpins GPU sales. The remaining headlines (SpaceX Nasdaq-100 addition, Fiserv, Robinhood, Microsoft restructuring, Buffett commentary, Hormuz shipping) are not material to NVDA's fundamentals. Net: no material change; the competitive-diversification theme continues to build slowly while demand signals stay firm.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>NVIDIA sits at the center of arguably the largest infrastructure buildout in tech history, nearly doubling revenue YoY while expanding margins -- a signature of demand exceeding supply and genuine pricing power. FCF generation is enormous (~$48.6B in a single quarter) with capex intensity under $2B/quarter, so growth converts to cash without heavy reinvestment. The CUDA software ecosystem creates switching costs that competitors must overcome across the full developer stack, not just raw hardware. Continued hyperscaler capex commitment -- reinforced today by Amazon's $25B AI-directed bond sale and robust high-bandwidth memory demand -- suggests the demand cycle has runway. At forward P/E ~15.4 and PEG ~0.6, the market implicitly prices meaningful deceleration; if the buildout persists even at a moderating pace, the stock is inexpensive relative to its own earnings trajectory. The fortress balance sheet (D/E ~0.06) and aggressive buybacks (financing outflows ~$21.3B latest quarter) provide downside cushion and shareholder-friendly capital return.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>The thesis rests entirely on the durability of hyperscaler AI capex, which is cyclical and concentrated among a few customers who are simultaneously NVIDIA's largest buyers and most motivated competitors. The steady drumbeat of customer diversification -- now including DeepSeek's own-chip effort alongside Turing/AMD shifts and growing TPU adoption -- is early but directionally real evidence that buyers want to reduce dependence and pricing leverage. Peak gross margins near 75% are difficult to defend indefinitely and naturally attract competition. Inventory more than doubled over the trailing period (from ~$11.3B to ~$25.8B), a risk of writedowns and margin compression if demand softens. A demand air pocket would hit NVIDIA disproportionately given the ~20% sequential growth now embedded in expectations. Beta of 2.2 means the stock amplifies any market drawdown, and a sentiment-driven repricing off a rich P/S (~19) and EV/EBITDA (~28) could be sharp. China export-control exposure remains an ongoing regulatory overhang. Finally, the latest quarter's 70%+ net margin exceeds the 65.6% operating margin, implying non-operating gains that may not recur and argue for normalizing earnings expectations down.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Financial health is exceptional on nearly every dimension and unchanged from the prior analysis. Revenue is high-quality and re-accelerating, with roughly three consecutive quarters of ~20% QoQ growth. Margins are best-in-class and trending up (gross ~75%, operating ~66%). Cash generation is outstanding: operating cash flow ~$50.3B and FCF ~$48.6B in the latest quarter (FCF margin ~60%). The balance sheet is fortress-like -- total debt ~$12.3B against ~$195.5B equity (D/E ~0.06), with immaterial leverage and very high interest coverage; current ratio ~3.4. Capital allocation favors shareholder returns via large buybacks and a token 0.5% dividend. Two items warrant monitoring rather than concern: inventory growth to ~$25.8B (a bet on future demand that becomes a markdown risk if demand softens) and elevated investing outflows (~$26-31B recent quarters, likely securities and strategic investments). ROIC ~77% and ROE ~82% remain among the highest of any large-cap.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Fairly Valued</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>The valuation picture is unchanged. On absolute multiples NVIDIA looks reasonable to cheap: forward P/E ~15.4 and PEG ~0.6 are undemanding for a business growing earnings at triple-digit YoY rates. Trailing P/E ~30 sits well below levels seen in prior enthusiasm phases, reflecting that earnings have caught up to the price. However, price-to-sales ~19 and EV/EBITDA ~28 are rich in absolute terms and only justified if current growth and margin structure persist. The crux: the attractive forward multiple embeds a large forward earnings estimate that itself depends on continued AI capex; if growth normalizes to a still-strong but decelerating pace, the forward multiple proves appropriate rather than a bargain. The stock trades at $196.93, roughly midway between its 52-week range ($158.39-$236.54), consistent with a market weighing quality against durability uncertainty. Given the exceptional business quality alongside genuine (if incremental) competitive and cyclical risks, 'Fairly Valued' remains the honest rating.</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>NVIDIA holds one of the strongest moats in technology, anchored by CUDA's software ecosystem and full-stack integration (GPUs, post-Mellanox networking, software), producing system-level lock-in and deep switching costs. Dominant AI-accelerator share sustains pricing power evident in ~75% gross margins. That moat is under measurable but still incremental pressure: AMD is gaining early credibility, hyperscalers' custom silicon (Google TPUs and others) represents structurally motivated in-house competition, and today's DeepSeek own-chip report adds another customer to the diversification list. The sheer profitability NVIDIA extracts is itself the strongest incentive for customers to develop alternatives. Switching costs are high but not absolute. The moat remains dominant today and is more likely to erode gradually than to break abruptly, but the accumulating list of customers pursuing in-house silicon is a trend worth tracking closely.</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>The multi-year growth runway remains strong: continued AI infrastructure buildout, scaling inference workloads as models reach production deployment, and expanding use cases (enterprise AI, sovereign AI, automotive/autonomy). Today's demand signals (Amazon capex, memory demand) support the near-term durability of the cycle. Ecosystem lock-in positions NVIDIA to capture the majority of accelerated-computing spend for the foreseeable future. The principal five-year risks are unchanged: (1) a cyclical demand correction if AI monetization lags capex, amplified by customer concentration; (2) gradual margin compression as AMD, TPUs, and now customers like DeepSeek building bespoke silicon capture share and gain pricing leverage; (3) regulatory/export constraints, particularly China. Base case is continued growth at a decelerating rate with some margin give-back from peak -- still an excellent outcome. Bear scenario is a demand air pocket plus faster competitive erosion. The outlook is robustly positive with wider-than-normal uncertainty bands.</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>NVIDIA is a rare combination of hypergrowth and exceptional profitability: ~85% YoY revenue growth, ~75% gross margins, ~77% ROIC, ~$49B quarterly FCF, and a near-debt-free balance sheet. At forward P/E ~15.4 and PEG ~0.6, the market prices meaningful deceleration, creating favorable asymmetry if the AI buildout persists even at a moderating pace. The core risks -- customer concentration, hyperscaler custom silicon, early AMD share gains, an expanding roster of customers (now including DeepSeek) building their own chips, peak margins, and cyclicality -- are real but continue to show incremental erosion, not structural breakdown. The CUDA ecosystem moat remains the decisive defensive asset, and today's news left the fundamental picture unchanged while adding balanced signals (one competitive negative, two demand positives). Net assessment: a high-quality, dominant franchise trading at a reasonable multiple for its growth, warranting a constructive but risk-aware stance. Valuation is fair rather than a bargain because the attractive forward multiple depends entirely on the durability of a demand cycle carrying genuine cyclical and competitive uncertainty. Position sizing should respect the high beta (2.2) and the risk of a sharp sentiment-driven repricing.</t>
+        </is>
+      </c>
+      <c r="M28" s="11" t="n">
+        <v>74</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Confidence is essentially unchanged from the prior writeup because no material new information arrived -- financials are identical and the news is incremental. It is supported by the clarity and strength of the financial data: growth, margins, cash generation, and returns on capital are unambiguous and exceptional, with no solvency concern. It is tempered by: the absence of Q4 2024/Q1 2025 financials limiting full trend analysis; the anomalous 70%+ net margin versus 65.6% operating margin, suggesting non-recurring items that cloud normalized earnings; and the biggest thesis variable -- the durability of AI capex and the pace of competitive erosion -- being inherently unforecastable. The DeepSeek own-chip news reinforces the diversification theme but is too small to quantify. The forward P/E's attractiveness depends on estimates I cannot independently verify from the data provided.</t>
+        </is>
+      </c>
+      <c r="O28" s="11" t="n">
+        <v>82</v>
+      </c>
+      <c r="P28" s="11" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>TSMC remains the world's dominant leading-edge foundry, and the financial data continues to show an exceptionally strong business. Q1 2026 revenue reached ~NT$1,134B, up ~35% year-over-year and ~8% sequentially, with diluted EPS of NT$110.4 (up ~58% YoY). Profitability sits at a series high: gross margin ~66.2%, operating margin ~58.1%, net margin ~50.5%, with ROIC ~46% and ROE ~32%. The balance sheet is fortress-like (debt/equity ~0.19 and declining, current ratio ~2.5, cash ~NT$3.0T) and the company self-funds ~NT$350B/quarter of capex while still generating ~NT$347B of free cash flow. This week's news flow is almost entirely thematic reinforcement of the AI demand narrative rather than any material fundamental change. At ~38x trailing and ~21x forward earnings, the stock is fairly priced for its growth-and-returns profile, with the primary un-hedgeable risk being geographic concentration in Taiwan. The investment case is essentially unchanged from the prior analysis.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Nothing materially changed since the prior writeup one day earlier. There are no new financial disclosures, and the fundamentals (margin inflection to ~66% gross / ~50% net, ~35% YoY revenue growth, ~46% ROIC) remain exactly as previously analyzed. The recent news is thematic and largely confirmatory: multiple items reiterate AI-driven demand durability (BofA's $1.5T enterprise AI spending framing, several 'AI beneficiary' pieces), and a couple note that customer diversification could broaden (a potential DeepSeek custom chip that would likely be fabricated by TSMC). A Samsung-driven semiconductor selloff is characterized as technical/momentum-driven rather than fundamental, and two ETF-construction articles simply underscore TSMC's centrality even when excluded from fabless-focused funds. None of these represent a change to the earnings power, competitive standing, or risk profile. The single most important fact remains the prior quarter's margin step-change, which is not new information here.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>TSMC is the structural chokepoint of the AI hardware buildout: essentially every leading fabless AI designer depends on its leading-edge nodes and CoWoS advanced packaging. The financials validate genuine pricing power — margins expanded to record levels even while capex stayed enormous, contradicting the 'capex crushes margins' fear. The combination of ~66% gross margin, ~50% net margin, ~46% ROIC and 30%+ revenue growth is rare at this scale. The moat is compounding: leading-edge fabs cost tens of billions and take years to ramp, and TSMC's process/yield lead deepens through multi-year customer co-design and high switching costs. Broadening demand (e.g., custom AI silicon from new entrants like DeepSeek, plus Marvell/Credo/Broadcom-type designers) means TSMC wins regardless of which chip designer prevails. The balance sheet funds all of this internally while still growing FCF, and a low-20s forward multiple is undemanding for this growth quality.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>The dominant risk is geopolitical concentration — the bulk of leading-edge capacity sits in Taiwan, and any cross-strait disruption would be catastrophic and cannot be hedged. Customer concentration is high, so an AI capex digestion phase or overbuild would hit TSMC disproportionately given semiconductor cyclicality; the ~35% YoY growth and record margins plausibly represent a cyclical high-water mark rather than a durable baseline. Rising structural capital intensity (~NT$350B/quarter capex) and lower-margin overseas fabs (US, Japan, Germany) could dilute the exceptional profitability shown here. Competitively, Intel Foundry and Samsung are deploying heavy capital and government subsidies; even partial success would pressure leading-edge pricing. The Samsung selloff this week is a reminder that memory/semiconductor sentiment can turn quickly. Finally, the stock trades near its 52-week high after a large rerating, so much good news is already priced and there is little cushion for disappointment.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Financial health is excellent and improving. Revenue has grown sequentially every quarter across the series, from ~NT$839B (Q1 2025) to ~NT$1,134B (Q1 2026), culminating in ~35% YoY growth. Margins expanded across every line (gross ~58.8% to ~66.2%, operating ~48.5% to ~58.1%, net ~43% to ~50.5%), signaling mix improvement and pricing power rather than one-off effects. Cash generation is robust: Q1 2026 operating cash flow of ~NT$699B against ~NT$352B capex yields ~NT$347B FCF, with cash rising to ~NT$3.0T. The balance sheet is conservative — debt/equity ~0.19 and steadily declining, current ratio ~2.5, quick ratio ~2.3. Returns on capital are outstanding (ROIC ~46%, ROE ~32%, ROA ~22%). Capital allocation is dominated by high-return reinvestment, which is appropriate; the dividend yield is modest (~0.8%) and there is no evident dilution. Note the valuation snapshot mixes NT$ financials with USD price data, making EV/EBITDA (~5.8) and price-to-book (~97x) unreliable as cross-currency figures; these should be treated cautiously.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Fairly Valued</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Trailing P/E of ~38x compresses to ~21x forward with a PEG of ~1.4, which must be judged against ~35% revenue growth, ~58% EPS growth, expanding margins, and ~46% ROIC. A low-20s forward multiple is not demanding for a business of this quality and growth — it is roughly in line with or below what the fundamentals justify, and the trailing-to-forward compression reflects expected continued earnings growth. The stock trades near the upper end of its 52-week range ($432.57 vs high $479, low $224), meaning much of the rerating has already occurred and a substantial amount of good news is priced in. Price-to-book (~97x) is not a useful bear signal given the accounting understates the earnings power of these assets and the currency mismatch distorts the figure. Balancing genuine fundamental acceleration against a full price and a likely cyclical peak in margins, 'Fairly Valued' remains the appropriate call — not a bargain, not an obvious short, with valuation risk concentrated in whether AI demand and record margins hold.</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>TSMC holds one of the widest moats in global manufacturing. It dominates leading-edge logic production and the advanced packaging (CoWoS) essential to AI accelerators. The moat rests on a compounding process/yield lead, enormous capital barriers to entry (leading-edge fabs cost tens of billions and years to ramp), deep multi-year co-engineering relationships with the largest fabless designers, and high switching costs once a design is tuned to a specific process. Pricing power is directly evidenced by margin expansion despite heavy capex. Industry structure at the leading edge is effectively an oligopoly narrowing toward a near-monopoly, with Samsung a distant second and Intel Foundry attempting re-entry with government backing. The potential broadening of the customer base (new custom-silicon designers such as DeepSeek routing to TSMC) reinforces its indispensability. The competitive threat from Intel/Samsung is real over a five-year horizon but unproven; TSMC's execution consistency remains a durable edge. The core structural vulnerability is geographic concentration in Taiwan, not competition.</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>The five-year outlook is strong on fundamentals with elevated tail risk. Growth drivers are secular: AI compute, high-performance computing, advanced packaging, and continued node migration all funnel through TSMC, and demand-side signals (enterprise AI adoption, sustained hyperscaler/fabless capex, broadening custom-silicon designs) point to a multi-year cycle rather than a short spike. Headwinds include inevitable semiconductor cyclicality (a demand digestion phase will come at some point), rising capital intensity, and margin drag from geographically diversified overseas fabs, plus intensifying competition from subsidized rivals. The overarching constraint is geopolitical concentration, which caps the multiple the market will pay regardless of operational excellence. Absent a geopolitical shock, TSMC should keep compounding revenue and earnings at attractive rates, though the record ~35% growth and ~66% gross margin of the latest quarter likely represent a high-water mark that normalizes over the cycle.</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>TSMC is a best-in-class business at a fair-but-not-cheap valuation, and nothing this week alters that. It is the indispensable manufacturer of leading-edge AI chips, with a moat evidenced by hard numbers rather than narrative — ~66% gross margin, &gt;50% net margin, ~46% ROIC, and 30%+ revenue growth, all while self-funding massive capex and de-levering a fortress balance sheet. At ~21x forward earnings with a PEG near 1.4, the market pays a reasonable price for durable, high-quality growth. The bull case is that AI demand proves structurally durable and TSMC's leading-edge monopoly sustains premium returns; the bear case is a geopolitical shock or a cyclical AI-capex digestion that reverses peak margins. This remains a high-conviction quality holding whose primary risk is exogenous (Taiwan) rather than operational or competitive. Appropriate posture is constructive ownership with position sizing that respects the un-hedgeable geopolitical tail risk, mindful that the stock trades near its 52-week high with much upside already priced.</t>
+        </is>
+      </c>
+      <c r="M29" s="11" t="n">
+        <v>76</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Confidence is supported by six quarters of consistent, mutually reinforcing financial data — accelerating revenue, margin expansion across every line, exceptional and stable returns on capital, and a de-leveraging balance sheet. These are hard facts, not sentiment, and the recent news is confirmatory rather than contradictory, so the thesis is stable. Confidence is limited by: (1) apparent currency/unit inconsistencies in the valuation snapshot (NT$ financials vs USD price) producing implausible EV and P/B figures, reducing precision on cross-currency multiples; (2) absence of ROE/ROIC for earlier quarters, limiting long-trend confirmation; (3) unquantifiable geopolitical tail risk that no financial analysis can price; and (4) the stock trading near its highs after a large rally, raising odds that near-term returns lag even if the business performs. Since this is only one day after the prior analysis with no material change, I hold the confidence level constant.</t>
+        </is>
+      </c>
+      <c r="O29" s="11" t="n">
+        <v>92</v>
+      </c>
+      <c r="P29" s="11" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Broadcom is a diversified semiconductor and infrastructure-software company riding a powerful AI-driven inflection. Across the five reported quarters, revenue accelerated from ~$15.0B (Q2 2025) to $22.2B (Q2 2026), with the latest quarter delivering ~48% YoY and ~15% sequential growth. Margins are exceptional and expanding: gross margins near 69%, operating margins climbing from ~39% to ~49%, and FCF margin of ~46% ($10.3B FCF on $22.2B revenue, on trivial ~$231M capex). The company generates enormous cash and continues deleveraging, with debt/equity falling from ~0.97 to ~0.74 and interest coverage rising to ~10.7x. ROE (~33%) and ROIC (~20%) confirm high-quality economics, though inflated by VMware's goodwill-heavy balance sheet. At ~$371 the stock trades at ~62x trailing and ~19x forward earnings, ~25% below its 52-week high of $495. This week's price action is a sentiment-driven pullback from a valuation downgrade, a broad chip selloff (Samsung guidance), and competitive-threat headlines (DeepSeek in-house chip), none of which alter the fundamentals in the data provided. The central tension remains a genuinely strong business against a valuation that leaves little room for disappointment.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Nothing in the underlying financials has changed since the prior analysis one day earlier; the reported quarterly data and ratios are identical. The material new items are all sentiment- and news-driven: (1) A valuation-based bank downgrade pushed shares down ~3% and reinforced the view that the stock is priced ahead of fundamentals rather than deteriorating. (2) A broad semiconductor selloff triggered by weak Samsung guidance and general risk-off macro pressure, again a sentiment reset rather than a company-specific event. (3) Reports that DeepSeek is developing its own AI inference chip, and that an Nvidia AI system slipped to 2028, which introduce two conflicting signals for AVGO's custom-ASIC franchise: on one hand, rising in-house/custom silicon efforts validate the ASIC/XPU merchant model Broadcom serves; on the other, a delayed Nvidia rack cycle could soften near-term demand for Broadcom's AI networking content and hyperscalers in-sourcing could pressure long-term share. These are incremental narrative developments, not a demonstrated change in Broadcom's order book or financials. My assessment and ratings are therefore essentially unchanged from the prior writeup.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Broadcom sits at the intersection of two secular franchises: custom AI accelerators (XPUs/ASICs) plus high-speed networking silicon, and a sticky infrastructure-software portfolio anchored by VMware, mainframe, and security. The financials show the thesis materializing: near-50% operating margins, ~46% FCF margins, and revenue reaccelerating to ~48% YoY reflect real operating leverage on a differentiated product set. Hyperscaler custom-silicon demand delivers high-margin, design-win-locked revenue with multi-year visibility, reinforced by the Apple extension through 2031. The software segment adds recurring, high-margin cash flow largely insulated from semiconductor cyclicality. Cash generation is prodigious and rising, funding continued deleveraging, dividends, and buybacks. A forward P/E of ~19x with a PEG near 0.4 implies that even partial persistence of growth makes the current price undemanding relative to the earnings trajectory. Notably, the proliferation of custom-silicon programs (including efforts like DeepSeek's) can validate rather than undermine Broadcom's merchant ASIC design model, since many such players still need Broadcom's IP, SerDes, and networking. ROIC ~20% and ROE ~33% mark a genuine compounder, not a commodity chipmaker.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>The valuation embeds continued hypergrowth: at ~62x trailing earnings, ~24x EV/revenue, and ~43x EV/EBITDA, any deceleration in AI/custom-silicon orders could compress the multiple sharply, as the ~25% drawdown from the 52-week high already hints. Custom-ASIC revenue is concentrated among a handful of hyperscaler customers whose capex plans can shift quickly; a reported Nvidia system delay to 2028 illustrates how AI infrastructure timelines can slip, potentially deferring Broadcom's networking content. Rising in-house AI chip efforts (DeepSeek and others) cut both ways and could over time reduce reliance on merchant partners for some workloads. The Q2 2026 inventory build (from $2.0B to $4.3B over the period, up sharply sequentially) warrants scrutiny as a possible demand-timing risk. Competition in AI optical interconnects and co-packaged optics is intensifying. The balance sheet still carries ~$65B of VMware-related debt, and book value is heavily goodwill/intangibles, so reported ROE/ROIC overstate tangible-capital returns. Quarterly net income is noisy (e.g., the tax/one-off-driven $8.5B in Q4 2025), making the trailing P/E an unreliable gauge.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Financial health is strong and improving. Revenue quality is high, blending design-win-locked semiconductor content with recurring software. Gross margin is stable near 68-69%; operating margin expanded from ~39% (Q2 2025) to ~49% (Q2 2026); FCF margin reached ~46% with $10.3B FCF on ~$231M capex, reflecting an asset-light, IP-driven model. Cash rose to ~$19.6B. The balance sheet carries ~$64.9B total debt against ~$87.7B equity (debt/equity ~0.74, down from ~0.97), with interest coverage improving to ~10.7x, clearly sustainable given cash generation. Financing outflows ($10.1B in Q1 2026, $4.8B in Q2 2026) are consistent with dividends, buybacks, and debt repayment; dividend yield is modest (~0.7%). Caveats: a large intangible/goodwill base from VMware inflates book-based returns, and the notable inventory increase in the latest quarter merits monitoring. Overall, this is a cash machine with a de-risking balance sheet.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Fairly Valued</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>The headline ~62x trailing P/E looks demanding but is distorted by uneven quarterly net income (including the large Q4 2025 figure). More informative are the ~19x forward P/E and PEG near 0.4, alongside ~43x EV/EBITDA and ~24x EV/revenue. For a business compounding revenue ~48% YoY with ~49% operating margins and ~46% FCF margins, a high-teens/low-20s forward multiple is not obviously excessive versus its own history for a franchise of this quality. This week's ~3% decline on a valuation downgrade and broad chip selloff is a sentiment reset, not a fundamental change; shares remain ~25% below the 52-week high. That said, the elevated EV/revenue and EV/EBITDA leave little margin for error if AI-driven growth decelerates or hyperscaler capex enters a digestion phase. Balancing exceptional cash economics and growth against a price that already discounts continued strong execution, Fairly Valued remains the most defensible rating.</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Broadcom holds a wide, durable moat across several niches. In custom silicon/ASICs, it is a leading merchant partner for hyperscalers building bespoke AI accelerators, a business with high switching costs because designs are co-engineered and multi-year (the Apple extension to 2031 exemplifies the stickiness). In high-speed networking (switching/routing, SerDes, optical), Broadcom is a share leader with deep IP and process advantages. The Infrastructure Software segment (VMware, mainframe, security) provides mission-critical, embedded products with strong renewal economics and pricing power, evident in ~69% gross margins and expanding operating margins. Threats include intensifying competition in AI optical interconnects/co-packaged optics and the concentration risk of serving a small set of hyperscalers who could in-source; the emergence of players developing their own inference chips (e.g., DeepSeek) is a reminder that in-sourcing is a live long-term risk even as it can also expand the merchant-ASIC market. On balance, IP moats, switching costs, and scale support a strong competitive position.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Over five years, the primary growth driver is AI infrastructure: custom accelerators and the networking backbone that connects them, where Broadcom's content per system is high and rising. Secondary drivers are the recurring, high-margin software franchise and steady non-AI demand across broadband, wireless, and enterprise. Industry tailwinds favor sustained data-center and AI capex, but this spending is cyclical and prone to digestion phases; the reported Nvidia system slip to 2028 is a concrete example of how deployment timelines can shift and introduce lumpiness. Key challenges include hyperscaler customer concentration, in-sourcing risk, rising competition in optical/networking, and execution/retention risk in the software business post-VMware. Given demonstrated margin expansion, cash generation, and deleveraging, the multi-year runway looks strong, but investors should expect volatility rather than smooth linear growth, with the outlook hinging on the durability of AI-driven demand.</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Broadcom is a high-quality compounder benefiting from a genuine AI-driven inflection: revenue reaccelerating to ~48% YoY, operating margins expanding to ~49%, ~46% FCF margins, and improving returns on capital (ROIC ~20%). Its moat rests on co-engineered custom silicon with multi-year design-win lock-in (reinforced by the Apple extension to 2031), leadership in high-speed networking, and a sticky software franchise generating recurring cash. The balance sheet is de-risking rapidly, with debt/equity down to ~0.74 and interest coverage above 10x. The offset is valuation: at ~19x forward earnings and ~24x EV/revenue, the market already prices in continued strong execution, leaving the stock vulnerable to AI-capex digestion or in-sourcing/competitive pressure, risks underscored by the inventory build, this week's sector selloff, an Nvidia timeline slip, and DeepSeek's in-house chip reports. The most reasonable stance is that this is a franchise worth owning at a fair (not cheap) price; long-term holders are compensated by quality and cash generation but should size positions with concentration and cyclicality risks in mind. Fairly Valued with a favorable long-term bias.</t>
+        </is>
+      </c>
+      <c r="M30" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Confidence rests on clear, consistent financial evidence: accelerating revenue, expanding margins, strong FCF, and a de-leveraging balance sheet, corroborated by the Apple extension and durable AI demand narrative. It is tempered by data gaps (Q4 2024/Q1 2025 are NaN, limiting multi-year trend analysis), a trailing P/E distorted by uneven quarterly net income, a goodwill-heavy balance sheet that inflates return ratios, and the absence of segment-level detail to isolate AI/custom-silicon economics from software. This week's news is directionally mixed (valuation downgrade and competitive threats versus AI-spend validation) and did not change the reported financials, so I hold confidence steady rather than raising or lowering it.</t>
+        </is>
+      </c>
+      <c r="O30" s="11" t="n">
+        <v>82</v>
+      </c>
+      <c r="P30" s="11" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>JPMorgan remains the largest and most diversified U.S. money-center bank, spanning Consumer &amp; Community Banking, an integrated Commercial &amp; Investment Bank, and Asset &amp; Wealth Management. The latest reported quarter (Q1 2026) showed genuine reacceleration: revenue of $49.8B (+~8.8% QoQ, +~9.9% YoY), net income of $16.5B, diluted EPS of $5.94 (+~17% YoY), net margin recovering to ~33% from the Q4 2025 trough of ~28%, and ROE in the healthy mid-teens (~16%). Shareholder equity has compounded steadily from $351B (Q1 2025) to $364B (Q1 2026) despite active buybacks, evidencing real internal capital generation. At ~16x trailing and ~14x forward earnings, ~2.6x book, and near its 52-week high ($339 vs. $343), the market already recognizes the franchise's quality. Recent news is largely non-material to fundamentals, with the notable exception of a possible consortium acquisition of a debit-card network (Fiserv's STAR) that could deepen JPM's payments infrastructure control. The core investment question is unchanged: whether current mid-teens ROE and ~33% margins are a durable run-rate or reflect a favorable point in the credit and capital-markets cycle. The provided data still lacks credit-provision, net-charge-off, CET1, and NIM detail — the key swing variables for a bank. Net, this is a premium franchise fairly priced for its quality.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Nothing in this cycle materially changes the thesis relative to the prior analysis; the financial data is identical (Q1 2026 remains the latest quarter), so the fundamental picture is unchanged. The most notable incremental item in the news flow is a report that JPMorgan and other large U.S. banks are exploring a joint acquisition of Fiserv's STAR debit network. This is worth flagging as a potential (not yet consummated) strategic move that would reduce JPM's reliance on third-party processors and strengthen its control over payments rails — economically sensible given its scale, though financial impact depends entirely on deal terms that are not disclosed. Other items (a BofA note anticipating strong Q2 bank earnings, robust IPO/listing demand such as SK Hynix, JPM's asset-management FX repositioning, and competitive ETF offerings) are directionally supportive of a favorable capital-markets and fee backdrop but are macro/non-specific and do not alter fundamentals. In short: no material change to the underlying thesis, one strategic optionality item to monitor.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>JPMorgan's scale, funding-cost advantage, and diversified earnings streams allow it to compound tangible book value through cycles while earning mid-teens ROE — a level most banks cannot sustainably reach. The integrated CIB captures advisory, underwriting, and trading revenue that is benefiting from a strong issuance and markets environment (evidenced by heavy listing demand and a supportive backdrop for Q2 bank earnings). Consumer banking supplies a low-cost, sticky deposit base and a large payments franchise generating durable net interest income, while AWM adds capital-light, fee-based earnings with high switching costs. Q1 2026's ~17% EPS growth and margin recovery to ~33% demonstrate operating leverage. The fortress balance sheet lets JPM take share opportunistically during stress. Consistent capital return — a ~10% dividend hike plus buybacks executed at a reasonable ~2.6x book — steadily supports per-share compounding. Potential vertical integration into payments infrastructure (the debit-network exploration) is a further margin/optionality lever. If capital-markets activity and rate normalization persist, earnings power looks resilient rather than peaking.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Bank earnings are inherently cyclical, and current ~33% net margins and mid-teens ROE may reflect a benign credit environment plus elevated capital-markets fees rather than a durable run-rate. The provided data gives no visibility into loan-loss reserves, provisions, or net charge-offs — a genuine analytical blind spot; a recession or credit normalization would raise provisions and compress earnings meaningfully. Net interest income is sensitive to the rate path; falling rates or deposit repricing could pressure margins. The Q4 2025 dip to ~28% net margin and $4.63 EPS shows quarterly volatility is real. Debt-to-equity has drifted up from ~1.34x (Q1 2025) to ~1.42x (Q1 2026), and operating cash flow swings violently ($120B in Q4 2025 to -$212B in Q1 2026), reflecting balance-sheet-driven flows that resist conventional analysis. At ~2.6x book and within ~1% of its 52-week high, much of the good news appears priced in, leaving limited margin of safety if the cycle turns. Regulatory capital requirements and perennial litigation/compliance costs remain overhangs.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Financial health is strong. Revenue has trended upward — roughly $45B/quarter through 2025 rising to $49.8B in Q1 2026 — and Q1 2026 net income of $16.5B is the highest in the observed window. Net margin of ~33% and ROE of ~16% indicate high-quality, profitable operations, though margin volatility is evident (28% in Q4 2025 vs. 33% in Q1 2026). Shareholder equity grew steadily from $351B to $364B across five quarters despite active buybacks, confirming genuine internal capital generation. Debt-to-equity of ~1.42x is normal for a large diversified bank though it has crept up modestly. Standard operating/free cash-flow metrics are not meaningful here — the large negative swings reflect changes in trading assets, loans, and deposits, not distress. Capital allocation is shareholder-friendly: a ~10% dividend increase (yield ~1.8%) plus ongoing buybacks near a reasonable book multiple. Key data gaps persist: no credit provisions, net charge-offs, CET1 ratio, NIM, or deposit trends, all central to fully assessing cycle resilience.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Fairly Valued</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>At ~16x trailing and ~14x forward earnings with price-to-book of ~2.6x on mid-teens ROE, JPM trades at the upper end of where large-cap banks historically clear. A 2.6x book multiple is defensible only if ROE stays sustainably in the mid-teens — which JPM has demonstrated but which is cyclically dependent. The forward P/E of ~14x embeds continued earnings growth consistent with the ~17% YoY EPS growth just posted, so the multiple is not stretched relative to demonstrated growth. However, the stock sits within ~1% of its 52-week high, so the market is already rewarding quality and momentum, offering little discount for cycle risk. This is a premium franchise fairly priced for its quality — not an obvious bargain but not expensive given proven returns on equity. I characterize it as fairly valued, leaning toward the high end of fair; the risk/reward is more attractive on cyclical weakness than at current levels.</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>JPMorgan has one of the widest moats in banking, rooted in scale, funding-cost advantage, diversification, technology investment, and brand. Its low-cost, sticky deposit base underpins a structural funding advantage, and the integrated CIB is a global leader in trading, underwriting, and advisory where scale and balance sheet directly drive share. High regulatory capital and compliance requirements act as barriers to entry favoring the largest, best-capitalized incumbents. Switching costs are meaningful in institutional/treasury services, custody, and wealth management. Pricing power is moderate — lending is largely commoditized — but breadth enables cross-selling and wallet-share capture. Potential vertical integration into payments infrastructure (the debit-network exploration) would further entrench its payments position. Relative to listed peers Visa and Mastercard (capital-light, higher-margin pure networks), JPM's moat is durable but its returns are structurally lower and more cyclical because it is a balance-sheet-intensive business.</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Over five years, JPMorgan's growth drivers include continued share gains from scale and technology investment, expansion in higher-margin, capital-light payments and asset/wealth management, and the ability to deploy its fortress balance sheet during stress. Industry tailwinds include ongoing digitalization and consolidation favoring the largest players. Headwinds include the inherent cyclicality of credit and capital markets, rate-path sensitivity, rising regulatory capital demands that cap returns, and fintech/non-bank competition in payments and lending. The demonstrated ability to earn mid-teens ROE and grow book value through varied environments supports a constructive but measured outlook: this is a steady compounder rather than a high-growth story. Earnings will fluctuate with the macro cycle, but franchise durability plus consistent capital return should support mid-single to high-single-digit long-term per-share value compounding.</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>JPMorgan is a best-in-class, diversified megabank that consistently earns mid-teens ROE, compounds tangible book value through cycles, and returns substantial capital via dividends and buybacks. The latest reported quarter confirms reaccelerating revenue and ~17% EPS growth with margin recovery, and the capital-markets backdrop remains supportive. The moat — scale, cheap deposits, regulatory barriers, and an integrated CIB — is durable, with optional upside from deeper payments-infrastructure integration. However, at ~2.6x book and ~14x forward earnings essentially at its 52-week high, the stock is fairly rather than attractively valued, and current profitability likely reflects a favorable point in the credit cycle. The provided data lacks credit-provision and capital-ratio visibility, the key swing factors for a bank. Net: a high-quality core financial holding suitable for long-term investors, best accumulated on cyclical weakness rather than at current elevated levels. Risk/reward is balanced, not compelling, today.</t>
+        </is>
+      </c>
+      <c r="M31" s="11" t="n">
+        <v>68</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Confidence is supported by clear, consistent financials showing strong and improving profitability (rising revenue, mid-teens ROE, growing equity, shareholder-friendly capital return) and a well-understood, durable business model. It is reduced by material data gaps: no credit-loss provisions, net charge-offs, CET1/capital ratios, or NIM/deposit detail — all essential for assessing cycle resilience. This cycle's news adds little of substance; the one item worth monitoring (the debit-network acquisition exploration) is unconfirmed and its financial impact is undisclosed. The cyclical nature of bank earnings and the stock's proximity to all-time highs continue to inject uncertainty into forward returns despite clear franchise quality. Confidence is unchanged from the prior analysis given no material fundamental change.</t>
+        </is>
+      </c>
+      <c r="O31" s="11" t="n">
+        <v>82</v>
+      </c>
+      <c r="P31" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Visa remains a structurally elite payment-network operator with financials that confirm a toll-booth economic model: gross margins above 81%, operating margins in the high-60s%, and net margins around 53-54% in the most recent quarters. Revenue rose from ~$9.6B (Q1 2025) to $11.2B (Q1 2026), with Q1 2026 up ~17% YoY and diluted EPS up ~35% YoY, showing both top-line acceleration and buyback-driven per-share leverage. Returns on capital are outstanding (ROE &gt;60%, ROIC ~45%, ROA ~23%), and interest coverage above 40x confirms low financial risk. The dominant news theme in the last week is competitive/thematic pressure from stablecoins and crypto rails (Circle/USDC volume dominance, regulated dirham stablecoin, Bitcoin ETF inflows) plus Mastercard's multi-rail expansion, set against countervailing pieces arguing Visa's steady volumes demonstrate resilience. None of these threats has yet dented Visa's numbers. At ~30.7x trailing and ~23.7x forward earnings and near the top of its 52-week range ($294-$365) at $352, the stock is priced for continued high-quality compounding with limited margin of safety. The core long-term question is unchanged: whether Visa's network moat withstands a multi-year migration to alternative rails while it keeps compounding volume and earnings.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>There is little materially new since the prior writeup one day earlier; the financial data set is identical, so no fundamental change has occurred. The news flow this week shifted emphasis toward stablecoin disintermediation specifically -- Circle's USDC reportedly running ~70% of stablecoin volume, a regulated dirham stablecoin launching on UAE exchanges, and strong crypto/Bitcoin ETF momentum -- which sharpens (but does not newly introduce) the alternative-rail threat already flagged. Notably, the prior analysis's reference to a potential bank consortium acquiring Fiserv's debit network does not reappear in this news set, so that specific threat is not corroborated here. Countervailing coverage frames Visa's steady ~15% revenue growth as evidence of resilience against crypto, and highlights Visa's own moves into agentic/AI commerce and stablecoin settlement. A technical breakout was noted but is trading-driven and not fundamentally meaningful. Net: no material change to fundamentals; the competitive narrative is more concentrated on stablecoins, which is a sentiment/framing shift rather than a numbers-level development.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Visa runs one of the highest-quality business models available: an asset-light, two-sided network on global electronic payments with ~81% gross, ~67-68% operating margins, and ~45% ROIC. The multi-decade secular shift from cash to digital and mobile payments continues to expand its transaction base without proportional cost growth, and Q1 2026's 17% YoY revenue and 35% YoY EPS growth show the franchise is still accelerating, not maturing. Aggressive buybacks (financing outflows of $6-9B in recent quarters) shrink the share count and amplify per-share economics. Visa is positioning at the center of emerging channels -- Visa Direct money movement, tokenization, AI-agent commerce, and even stablecoin settlement -- suggesting it can monetize new rails rather than only defend old ones; stablecoins can settle over Visa infrastructure rather than purely bypass it. A fortress balance sheet (interest coverage &gt;40x, debt/equity ~0.67) supports continued capital return and investment. Low beta (0.75) and highly predictable cash flows make it a resilient compounder through cycles.</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>The concentration of stablecoin and multi-rail headlines is a genuine long-term warning: if account-to-account, real-time payment, and blockchain/stablecoin rails scale, the card-network toll could be disintermediated, compressing the pricing power underpinning 50%+ net margins. Circle/USDC's dominance of stablecoin volume and regulated fiat-backed stablecoins launching in new jurisdictions show the alternative-rail ecosystem is maturing, and Mastercard's multi-rail diversification signals competitors preparing for a post-card world. Interchange regulation remains a persistent structural overhang on the entire card economic model. The stock's premium multiple (30.7x trailing) leaves little room for disappointment; any deceleration in volume or take-rate, or margin compression from competitive/regulatory forces, could de-rate the shares meaningfully given they sit near the 52-week high. The Q1 2026 FCF drop (FCF margin ~23% on $3.0B operating cash flow versus $6-7B typical) is likely timing but remains unexplained and should be confirmed as non-structural.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Financial health is excellent and unchanged. Revenue is high-quality and recurring, driven by transaction volume on a global network, with remarkably stable margins: gross ~81%, operating ~67-68%, net ~53-54% across recent quarters, indicating durable pricing power rather than cyclical strength. Cash generation is normally very strong (FCF margins 45-62%), though Q1 2026 dipped to ~23% on a $3.0B operating cash flow quarter versus the $6-7B norm -- this stands out and appears to be working-capital/timing rather than a deterioration in economics, but warrants monitoring. The balance sheet is solid: cash ~$12.4B, total debt ~$24B, debt/equity ~0.67, interest coverage &gt;40x. Capital allocation is shareholder-friendly, with heavy buybacks (financing outflows $6-9B/quarter) driving EPS growth ahead of net income growth, plus a modest dividend (~0.75% yield). Returns on capital are elite: ROE &gt;60%, ROIC ~45%, ROA ~23%.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Fairly Valued</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>At $352, Visa trades at ~30.7x trailing and ~23.7x forward earnings, EV/EBITDA ~22.7x, and PEG ~1.6 -- premium multiples that are consistent with Visa's own historical range for a franchise generating ~45% ROIC, 53%+ net margins, and 17% revenue growth with 35% EPS growth. A simplistic 'high P/E therefore overvalued' view is inappropriate given the durability and returns of the business; the forward P/E of ~23.7x against mid-teens revenue growth and higher EPS growth implies a reasonable growth-adjusted price. The shares sit near the upper end of their 52-week range ($294-$365), so there is limited margin of safety and the stock is not cheap. Weighing the strength and durability of the model against emerging (but unquantified) rail-competition risk, the valuation is fair -- appropriate compensation for quality, with downside if disintermediation begins to appear in volume or take-rate trends.</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Visa's moat is among the widest in financial services: a two-sided network of billions of cards and tens of millions of acceptance points, reinforced by network effects, entrenched brand acceptance, high switching costs for issuers and merchants, and a scaled, low-cost processing infrastructure (VisaNet). This yields exceptional pricing power, visible in 80%+ gross and 67%+ operating margins, within a rational effective duopoly with Mastercard. However, credible long-term erosion vectors are intensifying: stablecoin and crypto rails (USDC dominance, regulated fiat-backed stablecoins), real-time account-to-account systems, and Mastercard's multi-rail push. The offsetting nuance is that Visa can partly co-opt these -- settling stablecoin flows and extending Visa Direct/tokenization -- rather than being purely bypassed. None of these threats has yet materially dented volumes or margins, but they represent the first genuine structural challenges to the card-toll model in years.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>The five-year outlook remains favorable but with wider tail risk than Visa's history implies. Tailwinds: continued global cash-to-digital conversion, cross-border growth, Visa Direct money movement, tokenization, and monetization of new commerce channels including AI-agent purchasing and potentially stablecoin settlement. These support high-single to low-double-digit volume growth with margin stability and buyback-fueled EPS growth. Headwinds: persistent interchange regulation, maturing alternative rails (stablecoins, A2A/RTP) that could gradually compress value captured per transaction, and competitor diversification. The base case over five years is continued compounding, but the distribution of outcomes has widened -- investors should weight the possibility of slower growth and modest multiple compression if disintermediation accelerates faster than Visa's ability to monetize new rails.</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Visa is a best-in-class compounder: an asset-light payment network with elite margins (53%+ net), ~45% ROIC, accelerating revenue (17% YoY) and EPS (35% YoY) growth, a fortress balance sheet, and disciplined capital returns. Secular payment digitization continues to expand its transaction base, and it is proactively extending into money movement, tokenization, AI-driven commerce, and even stablecoin settlement. The primary risk is not near-term fundamentals -- which remain excellent -- but the longer-term structural threat of disintermediation from stablecoin/crypto and A2A rails and competitor multi-rail strategies, compounded by interchange regulation. At ~23.7x forward earnings and near its 52-week high, the stock is fairly valued: a full but justified price for quality, with limited margin of safety. The thesis is to own a durable compounder while monitoring whether emerging rail competition shows up in volume or take-rate trends, and to confirm the Q1 2026 FCF dip is timing-related. Net: a high-quality hold / accumulate-on-weakness rather than a bargain.</t>
+        </is>
+      </c>
+      <c r="M32" s="11" t="n">
+        <v>78</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Confidence is supported by the clarity and consistency of Visa's financials -- stable elite margins, high ROIC, strong balance sheet, and accelerating growth are unambiguous and grounded in the data. It is tempered by the absence of full ROE/ROIC history for early quarters, the unexplained Q1 2026 FCF drop, and the lack of financial data on peers (MA, JPM) to directly benchmark competitive share. The stablecoin/alternative-rail threats are genuinely material to the long-term moat but remain difficult to quantify from headlines, and this week's news added narrative emphasis without any change in the underlying numbers, so confidence is held steady rather than raised.</t>
+        </is>
+      </c>
+      <c r="O32" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="P32" s="11" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Mastercard remains one of the highest-quality business models in financial services, operating as one half of the global card-network duopoly with Visa. Reported financials continue to confirm elite economics: gross margins in the 76-79% range, operating margins around 58-60%, net margins consistently above 45%, and FCF margins that swing seasonally from ~30% in Q1 to over 60% in stronger quarters. The most recent quarter (Q1 2026) shows revenue of $8.40B, up ~15.8% YoY, with diluted EPS of $4.35, up ~21% YoY, alongside the usual Q1 sequential softness (-4.6% QoQ). The balance sheet carries ~$19B of debt against ~$8-11B cash, but interest coverage near 27-28x and ROIC near 90% underscore a capital-light, highly cash-generative model; negative-to-thin book equity and very high ROE/P/B are artifacts of aggressive buybacks, not distress. At ~30.8x trailing and ~23.3x forward earnings, the stock sits roughly in the lower-to-middle of its historical multiple range and ~12% below its 52-week high. The central long-term debate is unchanged: whether emerging payment rails (stablecoins, bank-owned debit networks) erode the card moat over a multi-year horizon. On balance the fundamentals remain exceptionally strong and the valuation is reasonable relative to quality and growth.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Nothing in this period materially changes the thesis; the news flow is largely a re-articulation of themes already identified in the prior analysis. The financial data set is unchanged from the previous writeup (same trailing quarters through Q1 2026), so there is no new fundamental data point to reassess. The most notable items are competitive-narrative developments rather than events: (1) Mastercard's participation in an open USD stablecoin initiative, which is a constructive signal that management is positioning to participate in, rather than be displaced by, stablecoin settlement rails; and (2) continued reporting that banks may pursue acquisition of a Fiserv-owned debit network, a genuine but still-early disintermediation threat. Neither has appeared in the financials. The stablecoin engagement is a modest incremental positive versus the prior analysis because it converts an abstract threat into a concrete strategic hedge, but it is directional messaging, not evidence of a fundamental shift. In short: no material change to the fundamental picture since the last analysis.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Mastercard is a duopoly network with powerful two-sided network effects, deeply embedded switching costs for issuers and merchants, and structural pricing power that is nearly impossible to replicate. It compounds revenue at double digits (Q1 2026 +15.8% YoY) while sustaining ~58-60% operating margins and converting a large share of revenue to free cash flow, with ROIC near 90%. The secular migration from cash to electronic payments, particularly in emerging markets and in commercial/B2B and cross-border flows, provides a multi-year growth runway. The value-added services layer (analytics, cybersecurity, consulting/AI, loyalty) grows faster than the core network, deepens customer entanglement, and diversifies away from pure interchange. Multi-rail expansion (Mastercard Move, virtual cards, and now stablecoin participation) positions the company to earn economics on newer flows rather than merely defend cards. Management's consistent, value-accretive buyback program ($3-5B financing outflows per quarter) amplifies per-share earnings. At ~23x forward earnings against 20%+ EPS growth, the risk/reward for a business of this quality is favorable.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>The most credible long-term risk remains disintermediation of card rails. A bank consortium acquiring a debit network (e.g., Fiserv's) could route volume around Mastercard, pressuring both transaction counts and pricing. Stablecoin/crypto settlement threatens near-zero-cost rails that could compress the disproportionately lucrative cross-border economics where Mastercard earns outsized margins; Mastercard joining a stablecoin initiative is a hedge but could also cannibalize higher-margin flows. Regulatory scrutiny of interchange is a persistent global overhang. The premium valuation (13.8x sales, 14.2x EV/revenue, 22.5x EV/EBITDA) leaves limited room for error, so any growth deceleration or margin erosion could trigger meaningful multiple compression. Revenue is exposed to consumer discretionary spending and is cyclically vulnerable in a downturn. The balance sheet is financially engineered for shareholder returns via buybacks that have produced thin/negative book equity, which works well only so long as cash generation stays robust. Concentration in a single business model raises idiosyncratic disruption risk over a 5-10 year horizon.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Financial health is excellent. Revenue is high-quality, recurring, and increasingly diversified across geographies and services, with consistent double-digit YoY growth (Q1 2026 +15.8%). Margins are elite and stable: gross margin ~76-79%, operating margin ~58-60%, net margin steady above 45% across all reported quarters. Cash generation is exceptional, with operating cash flow of $2.4B-$5.7B per quarter and FCF margins ranging from ~30% in seasonally weak Q1 to over 60% in Q3 2025. The balance sheet shows ~$19B total debt against ~$8-11B cash, but interest coverage near 27-28x makes debt comfortably serviceable. Reported debt-to-equity (~2.5-2.8x), very high ROE (&gt;190%), and P/B (~70x) are artifacts of buybacks that have shrunk book equity rather than signs of stress; ROIC near ~90% reflects an asset-light, capital-efficient model. Capital allocation strongly favors buybacks with a modest dividend (~0.65% yield), evidenced by $3-5B quarterly financing outflows (Q1 2026 financing outflow of ~$5.0B). The primary caution is that the thin/negative equity structure means the capital-return program depends on continued strong cash flows.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Fairly Valued</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>At ~30.8x trailing and ~23.3x forward earnings, Mastercard trades within its long-run historical range and toward the lower-to-middle portion of it; historically the stock has commanded 30-40x earnings given its growth and margin profile. The forward P/E of ~23.3x against 20%+ EPS growth implies a PEG near 1.64, which is not cheap but is justifiable for a duopoly compounder with ROIC near 90%. Price-to-sales of ~13.8x and EV/EBITDA of ~22.5x are high in absolute terms but consistent with the business's exceptional margins and cash conversion. The price sitting ~12% below the 52-week high suggests some multiple compression has already occurred. Given the combination of quality, growth, and a multiple modestly below historical peaks, the stock looks fairly valued with a slight lean toward attractive rather than expensive; it is not a deep-value situation, and the premium reflects genuine business quality rather than speculation. This rating is unchanged from the prior analysis, appropriately, since neither the financials nor the valuation inputs have materially shifted.</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Mastercard holds one of the widest and most durable moats available. As one half of the global card-network duopoly, it benefits from strong two-sided network effects, extremely high switching costs embedded in its rails, and structural pricing power. Industry structure is concentrated and rational, and the capital-light model delivers returns on capital that few businesses can match. Value-added services and multi-rail initiatives deepen customer entanglement and expand the addressable market. The principal threats are structural rather than from a single named competitor: bank-owned debit networks that could bypass the network, and stablecoin/crypto settlement rails that could undercut cross-border economics. Mastercard's decision to participate in an open USD stablecoin effort is evidence it intends to embed itself in emerging rails rather than defend cards alone, which modestly strengthens the case that it can participate in disruption. These threats are real but still nascent and have not appeared in the financials; the moat remains formidable while warranting ongoing monitoring.</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>The long-term outlook remains strong. Secular tailwinds include the continued global cash-to-digital migration, growth in commercial/B2B and cross-border flows, emerging-market penetration, and expansion of high-margin value-added services. Multi-rail and stablecoin initiatives are deliberate hedges that could turn disruptive settlement technologies into incremental revenue rather than pure threats. The chief headwinds are regulatory pressure on interchange, potential disintermediation from bank-owned networks, and stablecoin/crypto settlement that could compress the most lucrative cross-border economics over a 5-10 year horizon; success in offsetting these is not guaranteed and the landscape is more dynamic than a decade ago. Over the next five years the base case is continued double-digit revenue growth and mid-teens-plus EPS growth, with the pace potentially moderating if disruption accelerates or the consumer weakens cyclically.</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Mastercard is a best-in-class compounder: a duopoly network with elite and stable margins (net &gt;45%), extraordinary returns on capital (ROIC ~90%), consistent double-digit revenue growth, and prodigious free cash flow steadily deployed into buybacks. The financials show no deterioration, and the valuation at ~23x forward earnings against 20%+ EPS growth is reasonable relative to the company's own history and quality. The bull case rests on the enduring cash-to-digital shift, services diversification, and pricing power; the bear case rests on multi-year disintermediation risk from bank-owned debit rails and stablecoins alongside a premium multiple with limited margin for error. This period's news adds no material fundamental change—the stablecoin participation is a mild positive that converts an abstract threat into a concrete strategic hedge. On the evidence available, the moat and growth durability outweigh the still-early competitive threats, making Mastercard an attractive long-term holding for investors comfortable paying a quality premium, with disruption of the core rails the key variable to monitor.</t>
+        </is>
+      </c>
+      <c r="M33" s="11" t="n">
+        <v>78</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Confidence is high because the financial data is unusually clean and consistent: elite margins, strong cash generation, high interest coverage, and durable growth are directly evidenced across multiple quarters, and the duopoly moat is well established. It is unchanged from the prior analysis because no new financial data was introduced and the news flow reinforced rather than altered the existing thesis. Confidence is tempered by three factors: genuine early-stage structural threats (bank-owned debit networks, stablecoins) whose eventual impact is uncertain; the thin/negative book equity from buybacks that limits some traditional balance-sheet checks; and ratio fields (ROE, P/B) distorted by capital structure that require interpretation. Missing full-year segment detail and Q4 2024 comparability data slightly reduce precision.</t>
+        </is>
+      </c>
+      <c r="O33" s="11" t="n">
+        <v>90</v>
+      </c>
+      <c r="P33" s="11" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Amazon operates three engines -- North America retail, International retail, and AWS -- supplemented by high-margin advertising and Prime subscriptions. The trailing data through Q1 2026 shows a business scaling revenue past $180B/quarter with structurally improved profitability: operating margins now sit in the 11-13% range versus historically thin single-digit retail-era levels. Q1 2026 net income of $30.3B (16.7% net margin) and ~75% YoY EPS growth reflect strong operating leverage, but the headline was flattered by roughly $17B of non-operating items (EBIT of $40.6B vs operating income of $23.9B), so underlying operating momentum is more modest than the EPS print suggests. The defining strategic tension remains capital intensity: capex has ballooned to $39-44B per quarter to build AI/cloud infrastructure, pushing free cash flow negative in Q1 2026 (-$18.2B) despite robust operating cash flow. Amazon is now tapping the bond market for ~$25B to fund this buildout, and total debt has risen from ~$133B to ~$210B over the past year. ROIC of ~16-17% and ROE of ~20% suggest capital is still being deployed productively. Valuation at ~32x trailing and ~25x forward earnings sits within Amazon's historical norm for a franchise of this quality. Nothing in the last week materially changes the thesis established in the prior analysis.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>There is no material change from the previous analysis dated one day earlier. The only concrete news item -- the ~$25B bond sale to fund AI infrastructure -- was already identified and analyzed in the prior writeup, so it is not new. This week's news flow is otherwise repetitive coverage of the same bond-sale story (multiple outlets restating debt-funded AI capex), plus non-material or tangential items (DeepSeek's custom chip, SpaceX's Nasdaq-100 inclusion, Roku vs. Sirius XM, Trump crypto, a broad macro selloff on higher yields/oil). The DeepSeek custom-chip story is a mild, indirect positive that reinforces the industry-wide move toward proprietary AI silicon, validating Amazon's Trainium/Inferentia strategy, but it is directional color rather than a fundamental change. In short: no new quarter of financials, no new guidance, and no change to the balance-sheet or capex trajectory beyond what was already captured. Plainly stated, nothing material changed.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Amazon has transformed from a low-margin retailer into a diversified compound-margin business, with operating margins structurally higher (11-13%) than the sub-5% levels of a few years ago, driven by mix shift toward AWS, advertising, and third-party marketplace services -- high-margin, capital-light revenue layered on the retail base. AWS is the crown jewel: if the current AI infrastructure buildout captures meaningful enterprise AI/cloud workload share, incremental margins are very high and could sustain years of double-digit growth with expanding profitability. The company still generates enormous operating cash flow ($54.5B in Q4 2025, $26B in Q1 2026), so today's negative FCF reflects deliberate investment, not distress. ROIC of ~16-17% shows capital is still being deployed above its cost. The ability to raise $25B of debt cheaply reflects a fortress credit profile, funding growth without equity dilution. Revenue grew ~17% YoY in Q1 2026 -- a remarkable rate at this scale -- and the industry-wide push toward custom AI silicon (echoed by DeepSeek's chip effort) supports Amazon's own vertically integrated Trainium/Inferentia cost advantage.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>The AI capex cycle is the central risk. Capex of $39-44B per quarter has already driven FCF negative (-$18.2B in Q1 2026), and the $25B bond raise signals intensification. If AI/cloud demand disappoints or competitive pricing from Azure and Google Cloud compresses returns, Amazon could be left with a rapidly depreciating asset base, rising interest expense, and years of suppressed free cash flow. Total debt nearly doubled YoY to ~$210B, with long-term debt rising from ~$53B to ~$119B -- a material shift in balance-sheet risk profile, though still manageable. Earnings quality is a caveat: Q1 2026 net income substantially exceeded operating income on ~$17B of non-operating gains, so the ~75% EPS growth overstates operating momentum, and normalized earnings imply a higher effective multiple. Retail remains exposed to consumer-cyclical weakness, and macro pressure (higher yields, oil) can compress high-beta tech multiples (beta 1.46). At ~32x trailing earnings with FCF negative, the stock prices in continued flawless execution; any AWS growth stumble or capex-driven margin disappointment could de-rate the multiple.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Revenue quality is high and diversified, growing ~17% YoY to $181.5B in Q1 2026, with the best-margin revenue (AWS, advertising, subscriptions) carrying the strongest economics. Gross margin is stable at ~48-52%. Operating margin has improved to the 11-13% range -- a genuine structural gain. Operating cash flow is very strong ($26B in Q1 2026; $54.5B in Q4 2025), but free cash flow has turned sharply negative (-$18.2B in Q1 2026) as capex surged to $44B/quarter; this is investment-driven, not operational weakness. The balance sheet has weakened at the margin: total debt rose from ~$133B (Q1 2025) to ~$210B (Q1 2026), with a further ~$25B bond adding more. However, interest coverage remains very comfortable (~46x), debt-to-equity of ~0.47 is moderate against $442B of equity, and ~$102B of cash provides ample liquidity. ROE (~20%) and ROIC (~16-17%) indicate productive capital deployment. No dividend; share count is roughly flat, so dilution is not a concern and there is no evidence of meaningful buybacks. The key watch item remains whether rising capex and debt service continue to suppress free cash flow for an extended period.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Fairly Valued</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>At ~32x trailing and ~25x forward earnings, ~3.7x EV/revenue, and ~17.4x EV/EBITDA, Amazon trades within the range typical of its historically premium multiple for a high-growth franchise. For a business compounding revenue ~17% with expanding operating margins and mid-teens ROIC, a ~25x forward P/E is not demanding relative to its own history, where Amazon frequently commanded far higher multiples during retail-margin-compressed periods. Two factors temper enthusiasm: a PEG of ~1.83, and trailing earnings partly inflated by ~$17B of non-operating gains -- normalized operating earnings would push the effective multiple higher. Negative free cash flow makes FCF-based valuation unattractive today, but that reflects investment intensity rather than deteriorating economics. The stock sits ~12% below its 52-week high of $278.56 and well above its $196 low. Balancing a durable, improving franchise against elevated capex risk and somewhat flattered earnings, fairly valued is the most defensible conclusion -- neither an obvious bargain (despite media framing of 'historically cheap') nor stretched.</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Amazon possesses one of the widest moats in the market, spanning multiple businesses. In retail, its scale, logistics/fulfillment network, and Prime ecosystem create switching costs and a self-reinforcing marketplace flywheel that competitors struggle to replicate. AWS is a category leader in cloud infrastructure with deep switching costs (embedded enterprise workloads, data, and tooling), network effects, and pricing power from scale economics; its vertical integration into custom silicon (Trainium/Inferentia) is a structural cost advantage, reinforced by the broader industry shift toward proprietary AI chips. The advertising business benefits from proprietary purchase-intent data. Primary threats are Microsoft Azure and Google Cloud, where all three are spending aggressively on AI infrastructure -- a potential capacity arms race that could pressure returns. In retail, competition from Walmart and lower-cost cross-border platforms persists but has not eroded Amazon's dominance. Overall the moat is durable and multi-dimensional.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>The five-year outlook is anchored on AWS and AI. If Amazon successfully monetizes the AI infrastructure it is building, cloud can drive sustained double-digit growth with high incremental margins, while advertising continues scaling as a high-margin profit center. Retail provides a stable, cash-generative base with modest margin upside from automation and third-party mix. Tailwinds include secular cloud adoption, enterprise AI deployment, and Amazon's structural cost/logistics advantages. Headwinds include the risk that the current AI capex supercycle produces overcapacity or sub-cost-of-capital returns, intensifying cloud price competition, rising interest expense from a larger debt load, regulatory/antitrust scrutiny, and consumer-cyclical retail exposure. The realistic base case is continued mid-teens revenue growth with margins holding or gradually expanding, but with free cash flow suppressed for the next 1-3 years while the AI buildout is digested. Execution on capital allocation is the biggest swing variable.</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Amazon is a high-quality, multi-engine compounder whose profitability has structurally improved (operating margins now 11-13% vs low single digits historically) while still growing revenue ~17% at massive scale. The bull thesis rests on AWS and advertising continuing to shift the earnings mix toward high-margin, moaty businesses, with the current AI investment eventually earning strong returns given ~16-17% ROIC. The bear thesis centers on capital intensity: capex has driven FCF negative, debt nearly doubled to ~$210B, and a ~$25B bond raise signals more spending ahead -- if AI/cloud returns disappoint, free cash flow stays depressed and the premium multiple could compress. Earnings quality is a caveat, as Q1 2026 net income was materially boosted by non-operating gains. At ~25x forward earnings the stock is fairly valued for its quality and growth, offering reasonable but not exceptional risk-adjusted upside. This remains a hold/accumulate-on-weakness franchise for patient investors comfortable with a multi-year capex-digestion period, rather than a deep-value opportunity. The past week produced no fundamental change to this view.</t>
+        </is>
+      </c>
+      <c r="M34" s="11" t="n">
+        <v>68</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Confidence is supported by six quarters of consistent, high-quality financial data showing durable revenue growth, structurally improved margins, strong operating cash flow, and solid returns on capital, plus a clearly identifiable moat. It is reduced by: (1) missing full-year YoY comparability (several ratio fields are NaN and Q4 2024 data is absent), (2) earnings-quality concerns from large non-operating gains in Q1 2026, (3) genuine uncertainty about whether the aggressive AI capex cycle will earn its cost of capital -- the swing factor for the thesis, and (4) reliance on qualitative, largely repetitive news rather than fresh quantified data. Because nothing material changed this week, confidence is unchanged from the prior analysis.</t>
+        </is>
+      </c>
+      <c r="O34" s="11" t="n">
+        <v>88</v>
+      </c>
+      <c r="P34" s="11" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MCD</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>McDonald's remains a franchise-heavy, capital-light QSR operator with industry-leading and stable margins (operating margin consistently 44-48%, net margin ~30-33%) and strong free cash flow. The most recent reported quarter (Q1 2026) showed revenue of $6.52B, up ~9.4% YoY, net income of $1.98B, and EPS up ~6.9% YoY, confirming continued fundamental progress despite a soft QSR demand backdrop. The business carries a deliberately negative book equity (~-$1.29B) driven by years of debt-funded buybacks and dividends, a feature of its capital-return model rather than a distress signal given ~7.9x interest coverage and reliable operating cash flow. At $282, the stock trades ~17% below its 52-week high of $341.75 and near the low of $264.53, on ~23x trailing and ~20x forward earnings. This analysis covers a one-day increment (prior analysis dated 2026-07-07); the underlying financial data is unchanged, and news flow this week reinforces existing themes rather than introducing anything materially new. The picture remains a high-quality, wide-moat defensive compounder facing cyclical demand and intensifying value competition, priced at a full-but-fair valuation with no clear margin of safety.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Nothing materially changed since the prior analysis one day ago. No new quarterly financials, guidance, or capital-allocation actions were reported. This week's news is thematic reinforcement rather than fresh signal: several pieces frame MCD as a beaten-down dividend aristocrat and dividend-growth compounder (attractive to income investors after the pullback), while competition coverage centers on Wendy's digital/AI momentum and its recent stock rally, and one item favors Chipotle on valuation despite MCD's stronger traffic execution via the value menu. A former MCD HR executive moving to Kroger is operationally immaterial, and options-activity/'big move' speculation offers no fundamental read for long-term holders. Net: the core tension (resilient value-menu-driven traffic recovery versus broadening QSR/convenience competition and soft sector traffic) is unchanged from the prior writeup.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>MCD's franchise/royalty model produces durable, high-margin, capital-light cash flows -- operating margins consistently above 44% and net margins around 30-33% are among the best in the restaurant industry. The value-menu strategy is reviving traffic, evidenced by ~9.4% YoY revenue growth in Q1 2026 during a weak consumer environment, demonstrating brand pull and pricing discipline. Scale, owned real estate, global brand ubiquity, supply-chain purchasing power, and franchisee density create a wide, durable moat and make MCD the price-setter in value QSR. Low beta (0.42) and a dividend-aristocrat track record make it a defensive holding that can outperform in volatile or recessionary markets, aided by the trade-down effect that benefits value-oriented QSR. Free cash flow is robust (~$1.7B in Q1 2026) and supports continued dividend growth and buybacks. If MCD sustains mid-single-digit revenue and EPS growth while returning capital, it can deliver steady, lower-volatility total returns.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Competition is intensifying from multiple directions -- Wendy's digital/AI investment (and its recent ~28% one-month stock rally reflecting renewed momentum), convenience-store entrants into chicken/value, and broad QSR value wars -- which could erode traffic and force margin-dilutive promotions. The value-menu lever that is driving traffic may compress franchisee unit economics if discounting becomes structural rather than temporary. Sector-wide soft U.S. traffic points to cyclical pressure on the cost-conscious consumer base MCD depends on. Negative book equity and ~$54.9B total debt, while manageable at ~7.9x coverage, leave less cushion if cash flows weaken or rates stay elevated, and the current ratio hovering near 1.0 offers limited liquidity buffer. Growth is mature and mostly incremental, so multiple expansion is limited and the stock is sensitive to any deceleration. A PEG near 2.6 against ~7% EPS growth means investors are paying a quality premium with little embedded upside.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Revenue quality is high given the franchise-royalty-heavy model, producing stable recurring cash flows. Margins are excellent and stable across the last five reported quarters: gross margin ~56-58%, operating margin ~44-48%, net margin ~30-33%. Free cash flow is consistent ($1.25B-$2.42B quarterly; $1.73B in Q1 2026, FCF margin ~27%). The balance sheet shows negative shareholder equity (-$1.29B in Q1 2026), a deliberate result of cumulative buybacks and debt-funded distributions rather than operating losses. Total debt (~$54.9B) is substantial but supported by ~7.9x interest coverage and reliable operating cash flow (~$2.4B in Q1 2026). ROIC ~19% and ROA ~14% indicate efficient capital deployment; ROE is not meaningful given negative equity. Capital allocation prioritizes a growing dividend (~2.66% yield, aristocrat status) and buybacks. Watch items: current ratio near 1.0 and steadily widening negative equity (debt/equity moving from ~-15x to ~-43x over five quarters), which reduce financial flexibility.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Fairly Valued</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>At ~23x trailing and ~20x forward earnings, MCD trades within the range typical for a high-quality, wide-moat defensive compounder and ~17% below its 52-week high. EV/EBITDA of ~17x and price/sales of ~7.3x reflect a premium justified by best-in-class margins and cash conversion rather than an obvious excess. The forward P/E of ~20x against mid-single-digit EPS growth (~7% YoY) yields a PEG near 2.6, which is elevated and caps upside -- you are paying for quality and durability, not growth. Book-value metrics are not meaningful given negative equity. The pullback has brought the multiple to a reasonable level relative to MCD's own historical premium and business quality, but there is no clear margin of safety. A defensible entry for income/quality investors, but not a bargain.</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>McDonald's has one of the strongest moats in the restaurant industry, built on global scale, brand ubiquity, an extensive franchised real-estate footprint, supply-chain purchasing power, and cost leadership that confers pricing power and traffic resilience. The value-menu-driven traffic recovery in a weak consumer environment shows brand pull and price positioning remain intact. Switching costs are inherently low in QSR, so the moat rests on convenience density, marketing scale, and cost advantage rather than lock-in. Threats are real and broadening -- Wendy's digital/AI push, convenience-store entrants into value/chicken, and soft sector-wide traffic -- but few competitors can match MCD's cost structure, unit density, or global reach, keeping it the price-setter. The moat is wide and durable but not immune to margin pressure from persistent value competition.</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Over five years, growth drivers are international unit expansion, digital/loyalty and delivery monetization, and franchisee royalty growth on a mature but resilient base. The trade-down effect during economic softness structurally favors value-oriented QSR, benefiting MCD's positioning. Headwinds include intensifying competition across QSR and convenience channels, wage/input inflation for franchisees, and current sector-wide traffic softness. Expected growth is mid-single-digit at the revenue and EPS level, supplemented by dividends and buybacks to reach total returns. The central five-year challenge is defending traffic and value perception without permanently eroding franchise-level unit economics through discounting. The outlook is solid and defensive but not high-growth -- a compounder, not a breakout.</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>McDonald's is a wide-moat, capital-light, cash-generative franchise business trading at a full-but-fair valuation after a ~17% pullback. Q1 2026 confirms execution -- ~9.4% revenue growth and ~7% EPS growth in a soft consumer backdrop -- alongside industry-leading margins (~44% operating) and strong ROIC (~19%). The intentional negative-equity capital structure and ~$54.9B debt are supported by reliable free cash flow and ~7.9x interest coverage, funding a dividend-aristocrat payout and buybacks. The core risk is intensifying value competition (Wendy's digital momentum, convenience-store entrants, sector-wide traffic softness) that could pressure traffic and force margin-dilutive discounting. With a PEG near 2.6 and no meaningful margin of safety, this is best owned as a defensive quality holding for total return and downside protection (beta 0.42) rather than an aggressive alpha idea. The thesis: own a durable compounder at a reasonable price and collect a growing dividend, accepting mid-single-digit growth and limited multiple expansion. This one-day-later reassessment does not change that view.</t>
+        </is>
+      </c>
+      <c r="M35" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Confidence is supported by consistent financial evidence: stable high margins, strong FCF, solid ~19% ROIC, and manageable debt coverage across multiple quarters, plus a well-established moat and defensive characteristics. It is reduced by data gaps -- Q4 2024 financials are entirely NaN, YoY revenue/EPS growth is computable only for the most recent quarter, and comparable-store metrics and management guidance are absent. The competitive/demand picture is genuinely mixed (value-driven traffic recovery versus intensifying peer competition and sector-wide softness), and valuation offers no clear margin of safety. Because this increment covers only one additional day with no new fundamental data, confidence is unchanged from the prior analysis.</t>
+        </is>
+      </c>
+      <c r="O35" s="11" t="n">
+        <v>85</v>
+      </c>
+      <c r="P35" s="11" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>NIKE is the dominant global athletic footwear and apparel brand, currently working through a self-inflicted turnaround after a period of over-reliance on direct-to-consumer channels and weak product cadence. The stock trades at $43.21, near its 52-week low of $40 and roughly 46% below its 52-week high of $80.17, indicating the market has heavily de-rated the shares. Recent quarterly data show a business under margin pressure: gross margins have slipped from the low-42% range to about 40%, and operating margins have been volatile (2.9% to 8.1% across recent quarters). Revenue is essentially flat year-over-year (Q1 2026 up just 0.1% YoY), consistent with a stabilizing but not yet re-accelerating top line. The most recent reported diluted EPS of $0.72 (Q2 2026) suggests a meaningful sequential earnings recovery and represents strong YoY growth off a depressed prior-year base. Management has signaled a channel strategy reset—rebuilding wholesale relationships and cleaning inventory—which is the classic playbook for restoring healthy growth. The balance sheet remains solid with a current ratio above 2.0 and declining debt-to-equity (~0.79). The core question for a long-term holder is whether the brand's enduring pricing power and distribution reach can restore double-digit operating margins and mid-single-digit growth, which would make the current valuation attractive.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>This is the first writeup, so the following are the most material recent items. First, earnings appear to be inflecting: reported Q2 2026 diluted EPS of $0.72 is well above the $0.35 in Q1 2026 and prior quarters, and the earnings-beat coverage points to operational resilience. Second, management transition—a new CFO—introduces some uncertainty but is framed as continuity rather than disruption. Third, the strategic pivot back toward wholesale distribution and cleaner inventory is the most fundamentally important development: it directly addresses the primary cause of Nike's revenue and margin deterioration over the prior two years. Fourth, a 7-Eleven trademark lawsuit over shoe design is a minor legal item unlikely to be financially material for a company of this scale. Net: the operational data and strategy reset suggest the trough may be forming, though margins remain well below Nike's historical peak levels.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Nike remains arguably the strongest brand in its category globally, with unmatched scale, athlete/marketing budgets, and distribution. The turnaround thesis is credible: rebuilding wholesale partnerships and clearing excess inventory typically restores full-price sell-through and gross margins over 4-6 quarters. Gross margin is depressed at ~40% versus a historical range closer to 44-46%; even partial mean-reversion drives substantial EPS leverage. The stock has been cut nearly in half from its 52-week high, so if the company merely restores mid-single-digit revenue growth and recovers 200-400bps of operating margin, earnings power could expand meaningfully from the trough, and the forward P/E of ~18.5 would look cheap against restored earnings. The dividend yield of ~3.8% is well-supported and unusually high for Nike, offering downside cushion and signaling management confidence. Balance sheet strength (current ratio &gt;2, declining leverage) gives ample runway to fund the turnaround and continue buybacks/dividends. Q2 2026's EPS jump is early tangible evidence the recovery is underway.</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>The bear case, supported by the 'multi-year earnings deceleration' framing, is that Nike's problems are structural, not merely self-inflicted. Revenue is essentially flat YoY and margins have not durably recovered—Q1 2026 gross margin (40.2%) and operating margin (4.9%) both deteriorated sequentially from Q4 2025, showing the recovery is uneven. Competitive intensity in athletic footwear has risen materially, with newer performance and lifestyle brands taking share, particularly among younger and running-focused consumers, eroding Nike's pricing power. Greater China remains a chronic risk zone with weak consumer demand and local-brand competition. If the wholesale reset compresses margins (wholesale is structurally lower-margin than DTC), the margin recovery thesis could stall. The stock trading near 52-week lows may reflect a legitimate reassessment of Nike's terminal growth rate rather than temporary pessimism. A trailing P/E of ~20.6 on depressed earnings is not obviously cheap if earnings power has permanently reset lower.</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Nike's balance sheet is healthy. Cash of ~$6.7B, current ratio consistently above 2.0, and quick ratio around 1.4 indicate strong liquidity. Total debt (~$11.2B) against ~$14.1B equity gives debt-to-equity of ~0.79, which has trended down over the observed quarters—a positive deleveraging signal. Inventory has declined from ~$8.1B (Q3 2025) to ~$7.5B (Q1 2026), consistent with the stated cleanup effort. Profitability metrics are the concern: gross margin has slipped to ~40% from low-42%, and operating margin has been erratic (2.9%-8.1%), reflecting a business in transition. ROE of ~16-18% and ROIC of ~12-13% (per the two quarters reported) remain respectable for a consumer brand but are below Nike's historical premium levels. Net margins in the 4.6-6.4% range are subdued. Free cash flow data was not provided, limiting assessment of cash conversion, but the maintained ~3.8% dividend yield and prior buyback history suggest capital return remains active. Overall: strong balance sheet, weak-but-stabilizing profitability.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Fairly Valued</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>At $43.21, Nike trades at a trailing P/E of ~20.6 and forward P/E of ~18.5, with EV/EBITDA of ~14.6 and price-to-sales of ~1.38. These multiples sit below Nike's historical premium range (the stock historically commanded high-20s to 30s P/E during its growth heyday). However, the trailing earnings base is depressed by the turnaround, so the trailing P/E overstates cheapness on normalized earnings and understates it if margins recover. On a normalized-earnings view—assuming gross margin recovers toward 44% and operating margin toward 12%—the shares would look meaningfully undervalued. On a bear view where margins stay near current trough levels, the current multiple is roughly fair. Given genuine uncertainty about whether the margin reset is cyclical or structural, and price-to-sales of 1.38 being below the company's historical average, I rate it Fairly Valued with an upside skew. The ~3.8% dividend provides a valuation floor. This is not a bare 'P/E is high' assessment—it reflects the wide range of plausible normalized earnings.</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Nike possesses one of the strongest brand moats in consumer cyclicals, built on decades of marketing investment, athlete endorsements, iconic sub-brands (Jordan/Jumpman, Converse), and global distribution scale. Its pricing power historically supported gross margins in the mid-40s. However, the moat has narrowed: competitors have captured share in performance running and lifestyle categories, and Nike's DTC over-pivot damaged wholesale relationships that are now being rebuilt. Switching costs for consumers are essentially zero in footwear/apparel, so the moat rests entirely on brand equity and product innovation, both of which require constant reinvestment. The brand remains dominant but is no longer unassailable. The provided peer (GME) is not a meaningful competitive comparison. Overall, Nike still holds a wide but somewhat eroded moat—the key open question is whether recent share losses are temporary or reflect a durable shift in consumer preference.</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Over a five-year horizon, Nike's growth drivers include restored wholesale distribution, product innovation cadence, expanding campus/collegiate partnerships, international growth, and the structural tailwind of global athleisure and health/wellness trends. If management executes the reset, mid-single-digit revenue growth with margin recovery is achievable, producing solid EPS growth off the current trough. The primary risks are intensifying competition, chronic softness and local-brand encroachment in Greater China, and the possibility that DTC/wholesale mix shifts permanently cap margins below historical peaks. Macro discretionary spending sensitivity (beta 1.13) adds cyclicality. The most likely outcome is a gradual, multi-quarter recovery rather than a sharp snap-back, with meaningful execution risk. Nike is not structurally declining, but its era of premium growth-multiple expansion is likely behind it; the next five years are more about margin normalization and steady compounding than hypergrowth.</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Nike is a high-quality, dominant brand undergoing a self-inflicted turnaround that appears to be inflecting, trading near multi-year lows at a below-historical valuation. The core thesis is a margin-recovery and channel-reset story: gross margins are depressed at ~40% versus a historical mid-40s, and even partial normalization would drive substantial EPS leverage from a stabilized, flat revenue base. Early evidence (Q2 2026 EPS of $0.72, declining inventory, deleveraging balance sheet, wholesale rebuild) supports the turnaround, while a strong balance sheet and ~3.8% dividend limit downside. The bear risk is that competitive share losses and China weakness are structural rather than cyclical, in which case current earnings power is the new normal and the stock is only fairly valued. Given the balance of a stabilizing operational picture, a supportive valuation with upside optionality, and a defended dividend against genuine but not thesis-breaking competitive risks, this is an attractive risk/reward for a patient holder—but conviction is tempered by the unresolved question of margin durability. A moderate long position or accumulation on weakness is warranted, sized to reflect execution uncertainty.</t>
+        </is>
+      </c>
+      <c r="M36" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Confidence is moderate. It is increased by clear balance-sheet strength, tangible early turnaround signals (EPS inflection, inventory reduction, deleveraging), and a valuation that offers downside protection via the dividend. It is decreased by incomplete data (missing FCF, several NaN quarters, no historical multiple ranges provided), the erratic and still-depressed margin profile, flat revenue that has not yet demonstrated durable re-acceleration, and genuine ambiguity over whether competitive share losses are cyclical or structural. The mixed news signal (both 'turnaround ahead' and 'bear of the day/earnings deceleration') reflects the real disagreement in the evidence.</t>
+        </is>
+      </c>
+      <c r="O36" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="P36" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>